<commit_message>
Link added for #620
</commit_message>
<xml_diff>
--- a/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
+++ b/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cienacorp-my.sharepoint.com/personal/ndavis_ciena_com/Documents/Documents/WorkingDocuments/BluePlanet/ApiPo/Standards/TAPI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="261" documentId="8_{F9CDBA61-51EF-42D5-8F3D-8C6E9AD27539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4858701-0BE2-47B1-B994-DD84856EDC89}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFADF7CB-9027-4C8C-8BF3-B86C7AD6F261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
+    <workbookView xWindow="28725" yWindow="-16380" windowWidth="29040" windowHeight="16440" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="131">
   <si>
     <t>Feature</t>
   </si>
@@ -437,6 +437,9 @@
   </si>
   <si>
     <t>https://github.com/ietf-ivy-wg/network-inventory-yang</t>
+  </si>
+  <si>
+    <t>https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/onmi2025.ND.001-YangConfigStatements.pptx</t>
   </si>
 </sst>
 </file>
@@ -909,7 +912,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="100.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="71" style="1" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="9.140625" style="1"/>
@@ -1226,7 +1229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1265,7 +1268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>46</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>15</v>
       </c>
@@ -1572,6 +1575,9 @@
       <c r="F18" s="9" t="s">
         <v>80</v>
       </c>
+      <c r="G18" s="10" t="s">
+        <v>130</v>
+      </c>
       <c r="H18" s="1" t="s">
         <v>93</v>
       </c>
@@ -1592,7 +1598,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>30</v>
       </c>
@@ -1843,7 +1849,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>2</v>
       </c>
@@ -2526,7 +2532,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>48</v>
       </c>
@@ -2854,6 +2860,7 @@
     <hyperlink ref="G3" r:id="rId6" xr:uid="{B85E8F47-7893-459C-8DC1-8BC4AA02A23B}"/>
     <hyperlink ref="G4" r:id="rId7" xr:uid="{E38CDBF1-9601-4855-8DFD-AE8A6A3AD6BE}"/>
     <hyperlink ref="G7" r:id="rId8" xr:uid="{D578898C-48FA-4D82-82AF-E6661888BC34}"/>
+    <hyperlink ref="G18" r:id="rId9" xr:uid="{09D95B53-BA52-41E5-AAC0-0F3CBDC9FC82}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated during call 20250506
</commit_message>
<xml_diff>
--- a/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
+++ b/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cienacorp-my.sharepoint.com/personal/ndavis_ciena_com/Documents/Documents/WorkingDocuments/BluePlanet/ApiPo/Standards/TAPI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="386" documentId="8_{F9CDBA61-51EF-42D5-8F3D-8C6E9AD27539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BBB99DF-ACCB-4D6C-A79F-DA72E9940B63}"/>
+  <xr:revisionPtr revIDLastSave="403" documentId="8_{F9CDBA61-51EF-42D5-8F3D-8C6E9AD27539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9D5A6AD-D1CE-4EF4-870F-53062EADDE67}"/>
   <bookViews>
     <workbookView xWindow="-28875" yWindow="-16380" windowWidth="29040" windowHeight="16440" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="162">
   <si>
     <t>Feature</t>
   </si>
@@ -469,9 +469,6 @@
     <t>Add physical route to 2.1.3</t>
   </si>
   <si>
-    <t>Needed</t>
-  </si>
-  <si>
     <t>TIP request</t>
   </si>
   <si>
@@ -522,6 +519,26 @@
   </si>
   <si>
     <t>#626</t>
+  </si>
+  <si>
+    <t>#627</t>
+  </si>
+  <si>
+    <t>#628</t>
+  </si>
+  <si>
+    <t>#606
+#605
+#594</t>
+  </si>
+  <si>
+    <t>Relationship between TAPI, IETF, OC and CMIS</t>
+  </si>
+  <si>
+    <t>JS/ND</t>
+  </si>
+  <si>
+    <t>JS interop testing and OIF comments</t>
   </si>
 </sst>
 </file>
@@ -992,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -1036,7 +1053,7 @@
         <v>78</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>83</v>
@@ -1103,7 +1120,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>18</v>
       </c>
@@ -1118,6 +1135,9 @@
       </c>
       <c r="E3" s="2" t="s">
         <v>53</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>106</v>
@@ -1181,33 +1201,36 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>130</v>
+        <v>67</v>
       </c>
       <c r="C5" s="3">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>135</v>
+      <c r="D5" s="3">
+        <v>2.7</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>131</v>
+        <v>68</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="K5" s="1">
         <v>1</v>
       </c>
       <c r="L5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N5" s="1">
         <v>1</v>
@@ -1219,31 +1242,34 @@
     </row>
     <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>137</v>
+        <v>69</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>136</v>
+      <c r="D6" s="3">
+        <v>2.7</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>132</v>
+        <v>70</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="K6" s="1">
         <v>1</v>
       </c>
       <c r="L6" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N6" s="1">
         <v>1</v>
@@ -1253,30 +1279,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>134</v>
+      <c r="D7" s="3" t="s">
+        <v>135</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="K7" s="1">
         <v>1</v>
@@ -1285,40 +1305,40 @@
         <v>1</v>
       </c>
       <c r="M7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="1">
         <v>1</v>
       </c>
       <c r="O7" s="1">
         <f>K7*L7*M7*N7</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C8" s="3">
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="K8" s="1">
         <v>1</v>
       </c>
       <c r="L8" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="1">
         <v>2</v>
@@ -1328,27 +1348,33 @@
       </c>
       <c r="O8" s="1">
         <f>K8*L8*M8*N8</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C9" s="3">
         <v>1</v>
       </c>
-      <c r="D9" s="3">
-        <v>2.5</v>
+      <c r="D9" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>145</v>
+        <v>157</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="K9" s="1">
         <v>1</v>
@@ -1367,63 +1393,60 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="C10" s="3">
         <v>1</v>
       </c>
-      <c r="D10" s="3">
-        <v>2.7</v>
+      <c r="D10" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
       </c>
       <c r="L10" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="1">
         <v>1</v>
       </c>
       <c r="O10" s="1">
         <f>K10*L10*M10*N10</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C11" s="3">
         <v>1</v>
       </c>
       <c r="D11" s="3">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="K11" s="1">
         <v>1</v>
@@ -1444,10 +1467,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>47</v>
+        <v>145</v>
       </c>
       <c r="C12" s="3">
         <v>1</v>
@@ -1456,21 +1479,40 @@
         <v>2.7</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>155</v>
+        <v>53</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1</v>
+      </c>
+      <c r="L12" s="1">
+        <v>1</v>
+      </c>
+      <c r="M12" s="1">
+        <v>1</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1</v>
+      </c>
+      <c r="O12" s="1">
+        <f>K12*L12*M12*N12</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>7</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>82</v>
+        <v>67</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>152</v>
       </c>
       <c r="C13" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="3">
         <v>2.7</v>
@@ -1478,15 +1520,8 @@
       <c r="E13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="I13" s="10"/>
-      <c r="J13" s="1" t="s">
-        <v>88</v>
+      <c r="F13" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="K13" s="1">
         <v>1</v>
@@ -1507,49 +1542,30 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>9</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
+        <v>68</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="C14" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="3">
         <v>2.7</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="K14" s="1">
-        <v>1</v>
-      </c>
-      <c r="L14" s="1">
-        <v>2</v>
-      </c>
-      <c r="M14" s="1">
-        <v>1</v>
-      </c>
-      <c r="N14" s="1">
-        <v>1</v>
-      </c>
-      <c r="O14" s="1">
-        <f>K14*L14*M14*N14</f>
-        <v>2</v>
+        <v>154</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C15" s="3">
         <v>2</v>
@@ -1557,20 +1573,24 @@
       <c r="D15" s="3">
         <v>2.7</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>86</v>
+      <c r="E15" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>80</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="10"/>
       <c r="J15" s="1" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="K15" s="1">
         <v>1</v>
       </c>
       <c r="L15" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M15" s="1">
         <v>1</v>
@@ -1580,15 +1600,15 @@
       </c>
       <c r="O15" s="1">
         <f>K15*L15*M15*N15</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C16" s="3">
         <v>2</v>
@@ -1596,23 +1616,20 @@
       <c r="D16" s="3">
         <v>2.7</v>
       </c>
-      <c r="E16" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>60</v>
+      <c r="E16" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J16" s="8" t="s">
-        <v>91</v>
+        <v>87</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="K16" s="1">
         <v>1</v>
       </c>
       <c r="L16" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M16" s="1">
         <v>1</v>
@@ -1622,15 +1639,15 @@
       </c>
       <c r="O16" s="1">
         <f>K16*L16*M16*N16</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="C17" s="3">
         <v>2</v>
@@ -1638,38 +1655,38 @@
       <c r="D17" s="3">
         <v>2.7</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="5" t="s">
         <v>86</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="K17" s="1">
         <v>1</v>
       </c>
       <c r="L17" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M17" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N17" s="1">
         <v>1</v>
       </c>
       <c r="O17" s="1">
         <f>K17*L17*M17*N17</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="C18" s="3">
         <v>2</v>
@@ -1677,23 +1694,23 @@
       <c r="D18" s="3">
         <v>2.7</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>53</v>
+      <c r="E18" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>91</v>
       </c>
       <c r="K18" s="1">
         <v>1</v>
       </c>
       <c r="L18" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M18" s="1">
         <v>1</v>
@@ -1703,15 +1720,15 @@
       </c>
       <c r="O18" s="1">
         <f>K18*L18*M18*N18</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>53</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>58</v>
+        <v>45</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="C19" s="3">
         <v>2</v>
@@ -1720,16 +1737,22 @@
         <v>2.7</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>59</v>
+        <v>156</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="K19" s="1">
         <v>1</v>
       </c>
       <c r="L19" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M19" s="1">
         <v>2</v>
@@ -1739,15 +1762,15 @@
       </c>
       <c r="O19" s="1">
         <f>K19*L19*M19*N19</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>57</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>67</v>
+        <v>46</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="C20" s="3">
         <v>2</v>
@@ -1756,19 +1779,22 @@
         <v>2.7</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>68</v>
+        <v>53</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="K20" s="1">
         <v>1</v>
       </c>
       <c r="L20" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20" s="1">
         <v>1</v>
@@ -1778,15 +1804,15 @@
       </c>
       <c r="O20" s="1">
         <f>K20*L20*M20*N20</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
+        <v>53</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="C21" s="3">
         <v>2</v>
@@ -1795,22 +1821,19 @@
         <v>2.7</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="K21" s="1">
         <v>1</v>
       </c>
       <c r="L21" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M21" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N21" s="1">
         <v>1</v>
@@ -2384,47 +2407,38 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>1</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E36" s="5"/>
-      <c r="K36" s="1">
-        <v>2</v>
-      </c>
-      <c r="L36" s="1">
-        <v>3</v>
-      </c>
-      <c r="M36" s="1">
-        <v>1</v>
-      </c>
-      <c r="N36" s="1">
-        <v>5</v>
-      </c>
-      <c r="O36" s="1">
-        <f>K36*L36*M36*N36</f>
-        <v>30</v>
+        <v>69</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" s="3">
+        <v>3</v>
+      </c>
+      <c r="D36" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E37" s="5"/>
       <c r="K37" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L37" s="1">
         <v>3</v>
@@ -2437,58 +2451,55 @@
       </c>
       <c r="O37" s="1">
         <f>K37*L37*M37*N37</f>
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E38" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="E38" s="5"/>
       <c r="K38" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L38" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M38" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N38" s="1">
         <v>5</v>
       </c>
       <c r="O38" s="1">
         <f>K38*L38*M38*N38</f>
-        <v>40</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E39" s="5"/>
-      <c r="F39" s="1" t="s">
-        <v>71</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="E39" s="2"/>
       <c r="K39" s="1">
         <v>2</v>
       </c>
       <c r="L39" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M39" s="1">
         <v>2</v>
@@ -2498,55 +2509,58 @@
       </c>
       <c r="O39" s="1">
         <f>K39*L39*M39*N39</f>
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E40" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="E40" s="5"/>
+      <c r="F40" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="K40" s="1">
         <v>2</v>
       </c>
       <c r="L40" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M40" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N40" s="1">
         <v>5</v>
       </c>
       <c r="O40" s="1">
         <f>K40*L40*M40*N40</f>
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E41" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E41" s="2"/>
       <c r="K41" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L41" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M41" s="1">
         <v>1</v>
@@ -2556,29 +2570,26 @@
       </c>
       <c r="O41" s="1">
         <f>K41*L41*M41*N41</f>
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E42" s="2"/>
-      <c r="J42" s="1" t="s">
-        <v>103</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="E42" s="5"/>
       <c r="K42" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L42" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M42" s="1">
         <v>1</v>
@@ -2588,55 +2599,58 @@
       </c>
       <c r="O42" s="1">
         <f>K42*L42*M42*N42</f>
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E43" s="2"/>
+      <c r="J43" s="1" t="s">
+        <v>103</v>
+      </c>
       <c r="K43" s="1">
         <v>2</v>
       </c>
       <c r="L43" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M43" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N43" s="1">
         <v>5</v>
       </c>
       <c r="O43" s="1">
         <f>K43*L43*M43*N43</f>
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E44" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E44" s="2"/>
       <c r="K44" s="1">
         <v>2</v>
       </c>
       <c r="L44" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M44" s="1">
         <v>2</v>
@@ -2646,26 +2660,26 @@
       </c>
       <c r="O44" s="1">
         <f>K44*L44*M44*N44</f>
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E45" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="E45" s="5"/>
       <c r="K45" s="1">
         <v>2</v>
       </c>
       <c r="L45" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M45" s="1">
         <v>2</v>
@@ -2675,29 +2689,29 @@
       </c>
       <c r="O45" s="1">
         <f>K45*L45*M45*N45</f>
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E46" s="2"/>
       <c r="K46" s="1">
         <v>2</v>
       </c>
       <c r="L46" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M46" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N46" s="1">
         <v>5</v>
@@ -2709,14 +2723,14 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E47" s="2"/>
       <c r="K47" s="1">
@@ -2738,21 +2752,21 @@
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E48" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E48" s="2"/>
       <c r="K48" s="1">
         <v>2</v>
       </c>
       <c r="L48" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M48" s="1">
         <v>1</v>
@@ -2762,48 +2776,48 @@
       </c>
       <c r="O48" s="1">
         <f>K48*L48*M48*N48</f>
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E49" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="E49" s="5"/>
       <c r="K49" s="1">
         <v>2</v>
       </c>
       <c r="L49" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M49" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N49" s="1">
         <v>5</v>
       </c>
       <c r="O49" s="1">
         <f>K49*L49*M49*N49</f>
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E50" s="2"/>
       <c r="K50" s="1">
@@ -2813,26 +2827,26 @@
         <v>2</v>
       </c>
       <c r="M50" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N50" s="1">
         <v>5</v>
       </c>
       <c r="O50" s="1">
         <f>K50*L50*M50*N50</f>
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E51" s="2"/>
       <c r="K51" s="1">
@@ -2854,21 +2868,21 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E52" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E52" s="2"/>
       <c r="K52" s="1">
         <v>2</v>
       </c>
       <c r="L52" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M52" s="1">
         <v>1</v>
@@ -2878,26 +2892,26 @@
       </c>
       <c r="O52" s="1">
         <f>K52*L52*M52*N52</f>
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E53" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="E53" s="5"/>
       <c r="K53" s="1">
         <v>2</v>
       </c>
       <c r="L53" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M53" s="1">
         <v>1</v>
@@ -2907,26 +2921,26 @@
       </c>
       <c r="O53" s="1">
         <f>K53*L53*M53*N53</f>
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E54" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E54" s="2"/>
       <c r="K54" s="1">
         <v>2</v>
       </c>
       <c r="L54" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M54" s="1">
         <v>1</v>
@@ -2936,55 +2950,52 @@
       </c>
       <c r="O54" s="1">
         <f>K54*L54*M54*N54</f>
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>34</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C55" s="4"/>
+        <v>33</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C55" s="3"/>
       <c r="D55" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E55" s="2"/>
-      <c r="J55" s="1" t="s">
-        <v>117</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="E55" s="5"/>
       <c r="K55" s="1">
         <v>2</v>
       </c>
       <c r="L55" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M55" s="1">
         <v>1</v>
       </c>
       <c r="N55" s="1">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="O55" s="1">
         <f>K55*L55*M55*N55</f>
-        <v>198</v>
+        <v>30</v>
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C56" s="4"/>
       <c r="D56" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E56" s="2"/>
       <c r="J56" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K56" s="1">
         <v>2</v>
@@ -3005,72 +3016,75 @@
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>37</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C57" s="3"/>
+        <v>35</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C57" s="4"/>
       <c r="D57" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E57" s="2"/>
+      <c r="J57" s="1" t="s">
+        <v>118</v>
+      </c>
       <c r="K57" s="1">
         <v>2</v>
       </c>
       <c r="L57" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M57" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N57" s="1">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="O57" s="1">
         <f>K57*L57*M57*N57</f>
-        <v>40</v>
+        <v>198</v>
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C58" s="3"/>
       <c r="D58" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E58" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E58" s="2"/>
       <c r="K58" s="1">
         <v>2</v>
       </c>
       <c r="L58" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M58" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N58" s="1">
         <v>5</v>
       </c>
       <c r="O58" s="1">
         <f>K58*L58*M58*N58</f>
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E59" s="5"/>
       <c r="K59" s="1">
@@ -3092,20 +3106,16 @@
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E60" s="5"/>
-      <c r="H60" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="I60" s="10"/>
       <c r="K60" s="1">
         <v>2</v>
       </c>
@@ -3125,16 +3135,20 @@
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E61" s="5"/>
+      <c r="H61" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="I61" s="10"/>
       <c r="K61" s="1">
         <v>2</v>
       </c>
@@ -3154,14 +3168,14 @@
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E62" s="5"/>
       <c r="K62" s="1">
@@ -3183,21 +3197,21 @@
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C63" s="3"/>
       <c r="D63" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E63" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="E63" s="5"/>
       <c r="K63" s="1">
         <v>2</v>
       </c>
       <c r="L63" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M63" s="1">
         <v>1</v>
@@ -3207,26 +3221,26 @@
       </c>
       <c r="O63" s="1">
         <f>K63*L63*M63*N63</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C64" s="3"/>
       <c r="D64" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E64" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E64" s="2"/>
       <c r="K64" s="1">
         <v>2</v>
       </c>
       <c r="L64" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M64" s="1">
         <v>1</v>
@@ -3236,19 +3250,19 @@
       </c>
       <c r="O64" s="1">
         <f>K64*L64*M64*N64</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C65" s="3"/>
       <c r="D65" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E65" s="5"/>
       <c r="K65" s="1">
@@ -3269,92 +3283,87 @@
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A66" s="6">
-        <v>51</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C66" s="4"/>
+      <c r="A66" s="1">
+        <v>49</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C66" s="3"/>
       <c r="D66" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E66" s="7"/>
-      <c r="F66" s="6"/>
-      <c r="G66" s="6"/>
-      <c r="H66" s="6"/>
-      <c r="I66" s="6"/>
-      <c r="J66" s="1" t="s">
-        <v>109</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="E66" s="5"/>
       <c r="K66" s="1">
         <v>2</v>
       </c>
-      <c r="L66" s="6">
-        <v>1</v>
-      </c>
-      <c r="M66" s="6">
-        <v>1</v>
-      </c>
-      <c r="N66" s="6">
-        <v>99</v>
+      <c r="L66" s="1">
+        <v>3</v>
+      </c>
+      <c r="M66" s="1">
+        <v>1</v>
+      </c>
+      <c r="N66" s="1">
+        <v>5</v>
       </c>
       <c r="O66" s="1">
         <f>K66*L66*M66*N66</f>
-        <v>198</v>
+        <v>30</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A67" s="1">
-        <v>52</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C67" s="3"/>
+      <c r="A67" s="6">
+        <v>51</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C67" s="4"/>
       <c r="D67" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E67" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E67" s="7"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6"/>
+      <c r="H67" s="6"/>
+      <c r="I67" s="6"/>
+      <c r="J67" s="1" t="s">
+        <v>109</v>
+      </c>
       <c r="K67" s="1">
-        <v>1</v>
-      </c>
-      <c r="L67" s="1">
-        <v>3</v>
-      </c>
-      <c r="M67" s="1">
-        <v>1</v>
-      </c>
-      <c r="N67" s="1">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="L67" s="6">
+        <v>1</v>
+      </c>
+      <c r="M67" s="6">
+        <v>1</v>
+      </c>
+      <c r="N67" s="6">
+        <v>99</v>
       </c>
       <c r="O67" s="1">
         <f>K67*L67*M67*N67</f>
-        <v>15</v>
+        <v>198</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>55</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>63</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C68" s="3"/>
       <c r="D68" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E68" s="2"/>
-      <c r="F68" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>104</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="E68" s="5"/>
       <c r="K68" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L68" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M68" s="1">
         <v>1</v>
@@ -3364,25 +3373,31 @@
       </c>
       <c r="O68" s="1">
         <f>K68*L68*M68*N68</f>
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E69" s="2"/>
+      <c r="F69" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>104</v>
+      </c>
       <c r="K69" s="1">
         <v>2</v>
       </c>
       <c r="L69" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M69" s="1">
         <v>1</v>
@@ -3392,12 +3407,40 @@
       </c>
       <c r="O69" s="1">
         <f>K69*L69*M69*N69</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>59</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E70" s="2"/>
+      <c r="K70" s="1">
+        <v>2</v>
+      </c>
+      <c r="L70" s="1">
+        <v>2</v>
+      </c>
+      <c r="M70" s="1">
+        <v>1</v>
+      </c>
+      <c r="N70" s="1">
+        <v>5</v>
+      </c>
+      <c r="O70" s="1">
+        <f>K70*L70*M70*N70</f>
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T61" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O69">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O70">
       <sortCondition ref="C1:C61"/>
     </sortState>
   </autoFilter>
@@ -3415,9 +3458,9 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="H13" r:id="rId1" tooltip="otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" xr:uid="{DC8291FA-BBBC-4164-AFDF-A14D5C37779A}"/>
+    <hyperlink ref="H15" r:id="rId1" tooltip="otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" xr:uid="{DC8291FA-BBBC-4164-AFDF-A14D5C37779A}"/>
     <hyperlink ref="H26" r:id="rId2" tooltip="otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" xr:uid="{DA695823-06F7-4C4D-A0BB-56A71E8AB3AA}"/>
-    <hyperlink ref="H60" r:id="rId3" tooltip="otcc2023.ND.007_BasicPhysicalIntent.zip" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.007_BasicPhysicalIntent.zip" xr:uid="{73726784-3406-4A32-9F90-250F1899557B}"/>
+    <hyperlink ref="H61" r:id="rId3" tooltip="otcc2023.ND.007_BasicPhysicalIntent.zip" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.007_BasicPhysicalIntent.zip" xr:uid="{73726784-3406-4A32-9F90-250F1899557B}"/>
     <hyperlink ref="H23" r:id="rId4" tooltip="otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" xr:uid="{B1E96811-E3AB-4B6A-9B71-389668390DD1}"/>
     <hyperlink ref="H24" r:id="rId5" xr:uid="{39007AE4-376B-4AFF-B690-2B1FD75ED6B2}"/>
     <hyperlink ref="H25" r:id="rId6" xr:uid="{B85E8F47-7893-459C-8DC1-8BC4AA02A23B}"/>

</xml_diff>

<commit_message>
Updates to account for new issues/priorities
</commit_message>
<xml_diff>
--- a/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
+++ b/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cienacorp-my.sharepoint.com/personal/ndavis_ciena_com/Documents/Documents/WorkingDocuments/BluePlanet/ApiPo/Standards/TAPI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="403" documentId="8_{F9CDBA61-51EF-42D5-8F3D-8C6E9AD27539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9D5A6AD-D1CE-4EF4-870F-53062EADDE67}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7CCD126-8F49-4E8D-8D1F-2D2225682C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28875" yWindow="-16380" windowWidth="29040" windowHeight="16440" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="173">
   <si>
     <t>Feature</t>
   </si>
@@ -314,18 +314,12 @@
     <t>Was available for 2.5 but not implemented</t>
   </si>
   <si>
-    <t>Expected to be OK</t>
-  </si>
-  <si>
     <t>Both 547 and remainder of min/max value in YANG</t>
   </si>
   <si>
     <t>Significant history and complexity</t>
   </si>
   <si>
-    <t>Change to approach (and potential compatibility issue)</t>
-  </si>
-  <si>
     <t>Work under way in IETF. May cause changes in 2.7.</t>
   </si>
   <si>
@@ -345,9 +339,6 @@
   </si>
   <si>
     <t>May need to use any refinements to the approach in 2.7.</t>
-  </si>
-  <si>
-    <t>This is unlikely to deliver significant feature content in 2.7 but is necessary ground work for beyond 2.7.</t>
   </si>
   <si>
     <t>Potential feature delivery in 2.7</t>
@@ -500,9 +491,6 @@
     <t>Draft YANG ready</t>
   </si>
   <si>
-    <t>Confirmed</t>
-  </si>
-  <si>
     <t>Sketch available</t>
   </si>
   <si>
@@ -539,6 +527,74 @@
   </si>
   <si>
     <t>JS interop testing and OIF comments</t>
+  </si>
+  <si>
+    <t>#629</t>
+  </si>
+  <si>
+    <t>ND/RC/RJ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Specific work on multiple service request.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+This is unlikely to deliver significant feature content in 2.7 but is necessary ground work for beyond 2.7.</t>
+    </r>
+  </si>
+  <si>
+    <t>Change to approach (and potential compatibility issue)
+Discussion underway. Will report back on calls.</t>
+  </si>
+  <si>
+    <t>TAPI Notification API Clarificaton</t>
+  </si>
+  <si>
+    <t>#631</t>
+  </si>
+  <si>
+    <t>Needs prioritization</t>
+  </si>
+  <si>
+    <t>Event Object Notification attribute target-object-dri to be classified as conditional attribute</t>
+  </si>
+  <si>
+    <t>2.5
+2.6
+2.7</t>
+  </si>
+  <si>
+    <t>#632</t>
+  </si>
+  <si>
+    <t>Expected to be OK. Confirmed.</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>#633</t>
+  </si>
+  <si>
+    <t>#634</t>
+  </si>
+  <si>
+    <t>#635</t>
   </si>
 </sst>
 </file>
@@ -602,7 +658,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -621,6 +677,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -635,7 +703,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -669,6 +737,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1009,7 +1089,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
-  <dimension ref="A1:O70"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:O72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -1038,13 +1119,13 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>56</v>
@@ -1053,7 +1134,7 @@
         <v>78</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>83</v>
@@ -1074,121 +1155,86 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
+        <v>70</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>71</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <v>15</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="3">
-        <v>1</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3">
         <v>2.7</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="E4" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="I2" s="10"/>
-      <c r="J2" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="K2" s="1">
-        <v>1</v>
-      </c>
-      <c r="L2" s="1">
-        <v>3</v>
-      </c>
-      <c r="M2" s="1">
-        <v>1</v>
-      </c>
-      <c r="N2" s="1">
-        <v>1</v>
-      </c>
-      <c r="O2" s="1">
-        <f>K2*L2*M2*N2</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>18</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="3">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3">
-        <v>2.7</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1</v>
-      </c>
-      <c r="L3" s="1">
-        <v>2</v>
-      </c>
-      <c r="M3" s="1">
-        <v>1</v>
-      </c>
-      <c r="N3" s="1">
-        <v>1</v>
-      </c>
-      <c r="O3" s="1">
-        <f>K3*L3*M3*N3</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>54</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="3">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>62</v>
-      </c>
+      <c r="H4" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="I4" s="10"/>
       <c r="J4" s="1" t="s">
-        <v>90</v>
+        <v>161</v>
       </c>
       <c r="K4" s="1">
         <v>1</v>
       </c>
       <c r="L4" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M4" s="1">
         <v>1</v>
@@ -1198,15 +1244,15 @@
       </c>
       <c r="O4" s="1">
         <f>K4*L4*M4*N4</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>57</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>67</v>
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="C5" s="3">
         <v>1</v>
@@ -1215,13 +1261,16 @@
         <v>2.7</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>105</v>
+        <v>154</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>84</v>
       </c>
       <c r="K5" s="1">
         <v>1</v>
@@ -1242,25 +1291,25 @@
     </row>
     <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
       </c>
-      <c r="D6" s="3">
-        <v>2.7</v>
+      <c r="D6" s="3" t="s">
+        <v>132</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="K6" s="1">
         <v>1</v>
@@ -1279,33 +1328,36 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>130</v>
+        <v>67</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>135</v>
+      <c r="D7" s="3">
+        <v>2.7</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>131</v>
+        <v>68</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="K7" s="1">
         <v>1</v>
       </c>
       <c r="L7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N7" s="1">
         <v>1</v>
@@ -1315,33 +1367,36 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>137</v>
+        <v>69</v>
       </c>
       <c r="C8" s="3">
         <v>1</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>136</v>
+      <c r="D8" s="3">
+        <v>2.7</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>132</v>
+        <v>70</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="K8" s="1">
         <v>1</v>
       </c>
       <c r="L8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="1">
         <v>1</v>
@@ -1351,30 +1406,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C9" s="3">
         <v>1</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>134</v>
+      <c r="D9" s="3" t="s">
+        <v>132</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="K9" s="1">
         <v>1</v>
@@ -1383,40 +1432,40 @@
         <v>1</v>
       </c>
       <c r="M9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="1">
         <v>1</v>
       </c>
       <c r="O9" s="1">
         <f>K9*L9*M9*N9</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C10" s="3">
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
       </c>
       <c r="L10" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="1">
         <v>2</v>
@@ -1426,27 +1475,33 @@
       </c>
       <c r="O10" s="1">
         <f>K10*L10*M10*N10</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C11" s="3">
         <v>1</v>
       </c>
-      <c r="D11" s="3">
-        <v>2.5</v>
+      <c r="D11" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>144</v>
+        <v>153</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="K11" s="1">
         <v>1</v>
@@ -1465,63 +1520,60 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C12" s="3">
         <v>1</v>
       </c>
-      <c r="D12" s="3">
-        <v>2.7</v>
+      <c r="D12" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="K12" s="1">
         <v>1</v>
       </c>
       <c r="L12" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N12" s="1">
         <v>1</v>
       </c>
       <c r="O12" s="1">
         <f>K12*L12*M12*N12</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="C13" s="3">
         <v>1</v>
       </c>
       <c r="D13" s="3">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="K13" s="1">
         <v>1</v>
@@ -1542,10 +1594,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>47</v>
+        <v>142</v>
       </c>
       <c r="C14" s="3">
         <v>1</v>
@@ -1554,21 +1606,40 @@
         <v>2.7</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>154</v>
+        <v>53</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1</v>
+      </c>
+      <c r="L14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>1</v>
+      </c>
+      <c r="N14" s="1">
+        <v>1</v>
+      </c>
+      <c r="O14" s="1">
+        <f>K14*L14*M14*N14</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>7</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>82</v>
+        <v>67</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="C15" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="3">
         <v>2.7</v>
@@ -1576,15 +1647,8 @@
       <c r="E15" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="I15" s="10"/>
-      <c r="J15" s="1" t="s">
-        <v>88</v>
+      <c r="F15" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="K15" s="1">
         <v>1</v>
@@ -1605,70 +1669,58 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>9</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>7</v>
+        <v>68</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="C16" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="3">
         <v>2.7</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="K16" s="1">
-        <v>1</v>
-      </c>
-      <c r="L16" s="1">
-        <v>2</v>
-      </c>
-      <c r="M16" s="1">
-        <v>1</v>
-      </c>
-      <c r="N16" s="1">
-        <v>1</v>
-      </c>
-      <c r="O16" s="1">
-        <f>K16*L16*M16*N16</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C17" s="3">
+        <v>2</v>
+      </c>
+      <c r="C17" s="13">
         <v>2</v>
       </c>
       <c r="D17" s="3">
         <v>2.7</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>86</v>
+        <v>53</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>158</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>80</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="I17" s="10"/>
       <c r="J17" s="1" t="s">
-        <v>98</v>
+        <v>160</v>
       </c>
       <c r="K17" s="1">
         <v>1</v>
       </c>
       <c r="L17" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M17" s="1">
         <v>1</v>
@@ -1678,15 +1730,15 @@
       </c>
       <c r="O17" s="1">
         <f>K17*L17*M17*N17</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="C18" s="3">
         <v>2</v>
@@ -1694,23 +1746,27 @@
       <c r="D18" s="3">
         <v>2.7</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>86</v>
+      <c r="E18" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>60</v>
+        <v>170</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>91</v>
+        <v>76</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="I18" s="10"/>
+      <c r="J18" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="K18" s="1">
         <v>1</v>
       </c>
       <c r="L18" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M18" s="1">
         <v>1</v>
@@ -1720,15 +1776,15 @@
       </c>
       <c r="O18" s="1">
         <f>K18*L18*M18*N18</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="C19" s="3">
         <v>2</v>
@@ -1737,16 +1793,16 @@
         <v>2.7</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="K19" s="1">
         <v>1</v>
@@ -1755,22 +1811,22 @@
         <v>2</v>
       </c>
       <c r="M19" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N19" s="1">
         <v>1</v>
       </c>
       <c r="O19" s="1">
         <f>K19*L19*M19*N19</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>41</v>
+        <v>74</v>
       </c>
       <c r="C20" s="3">
         <v>2</v>
@@ -1778,23 +1834,23 @@
       <c r="D20" s="3">
         <v>2.7</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>53</v>
+      <c r="E20" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>172</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>149</v>
+        <v>80</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="K20" s="1">
         <v>1</v>
       </c>
       <c r="L20" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M20" s="1">
         <v>1</v>
@@ -1804,15 +1860,15 @@
       </c>
       <c r="O20" s="1">
         <f>K20*L20*M20*N20</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>53</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>58</v>
+        <v>31</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="C21" s="3">
         <v>2</v>
@@ -1820,35 +1876,41 @@
       <c r="D21" s="3">
         <v>2.7</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>110</v>
+      <c r="E21" s="5" t="s">
+        <v>86</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>90</v>
       </c>
       <c r="K21" s="1">
         <v>1</v>
       </c>
       <c r="L21" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M21" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N21" s="1">
         <v>1</v>
       </c>
       <c r="O21" s="1">
         <f>K21*L21*M21*N21</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>60</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>111</v>
+        <v>45</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="C22" s="3">
         <v>2</v>
@@ -1856,60 +1918,65 @@
       <c r="D22" s="3">
         <v>2.7</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>53</v>
+      <c r="E22" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="K22" s="1">
         <v>1</v>
       </c>
       <c r="L22" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M22" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N22" s="1">
         <v>1</v>
       </c>
       <c r="O22" s="1">
         <f>K22*L22*M22*N22</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="C23" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D23" s="3">
         <v>2.7</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="2" t="s">
         <v>53</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="I23" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>169</v>
+      </c>
       <c r="J23" s="1" t="s">
-        <v>100</v>
+        <v>168</v>
       </c>
       <c r="K23" s="1">
         <v>1</v>
       </c>
       <c r="L23" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M23" s="1">
         <v>1</v>
@@ -1919,102 +1986,91 @@
       </c>
       <c r="O23" s="1">
         <f>K23*L23*M23*N23</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>5</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>5</v>
+        <v>53</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>58</v>
       </c>
       <c r="C24" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D24" s="3">
         <v>2.7</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H24" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="I24" s="11"/>
-      <c r="J24" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
       <c r="K24" s="1">
         <v>1</v>
       </c>
       <c r="L24" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M24" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N24" s="1">
         <v>1</v>
       </c>
       <c r="O24" s="1">
         <f>K24*L24*M24*N24</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>8</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>126</v>
+        <v>60</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="C25" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" s="3">
         <v>2.7</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="G25" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="I25" s="11"/>
       <c r="J25" s="1" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="K25" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L25" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M25" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" s="1">
         <v>1</v>
       </c>
       <c r="O25" s="1">
         <f>K25*L25*M25*N25</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C26" s="3">
         <v>3</v>
@@ -2022,42 +2078,42 @@
       <c r="D26" s="3">
         <v>2.7</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G26" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H26" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="I26" s="10"/>
+      <c r="G26" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="I26" s="11"/>
       <c r="J26" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="K26" s="1">
         <v>1</v>
       </c>
       <c r="L26" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M26" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N26" s="1">
         <v>1</v>
       </c>
       <c r="O26" s="1">
         <f>K26*L26*M26*N26</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>10</v>
+        <v>123</v>
       </c>
       <c r="C27" s="3">
         <v>3</v>
@@ -2072,14 +2128,14 @@
         <v>73</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I27" s="11"/>
       <c r="J27" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K27" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L27" s="1">
         <v>2</v>
@@ -2097,10 +2153,10 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C28" s="3">
         <v>3</v>
@@ -2108,20 +2164,24 @@
       <c r="D28" s="3">
         <v>2.7</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="5" t="s">
         <v>53</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>107</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="I28" s="10"/>
       <c r="J28" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="K28" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L28" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M28" s="1">
         <v>1</v>
@@ -2131,15 +2191,15 @@
       </c>
       <c r="O28" s="1">
         <f>K28*L28*M28*N28</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C29" s="3">
         <v>3</v>
@@ -2147,32 +2207,42 @@
       <c r="D29" s="3">
         <v>2.7</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>55</v>
+      <c r="E29" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="I29" s="11"/>
+      <c r="J29" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="K29" s="1">
         <v>1</v>
       </c>
       <c r="L29" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M29" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N29" s="1">
         <v>1</v>
       </c>
       <c r="O29" s="1">
         <f>K29*L29*M29*N29</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="C30" s="3">
         <v>3</v>
@@ -2183,35 +2253,35 @@
       <c r="E30" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>73</v>
+      <c r="G30" s="1" t="s">
+        <v>104</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="K30" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L30" s="1">
         <v>2</v>
       </c>
       <c r="M30" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N30" s="1">
         <v>1</v>
       </c>
       <c r="O30" s="1">
         <f>K30*L30*M30*N30</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="C31" s="3">
         <v>3</v>
@@ -2220,37 +2290,31 @@
         <v>2.7</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="K31" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L31" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M31" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" s="1">
         <v>1</v>
       </c>
       <c r="O31" s="1">
         <f>K31*L31*M31*N31</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="C32" s="3">
         <v>3</v>
@@ -2264,15 +2328,11 @@
       <c r="G32" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H32" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="I32" s="11"/>
       <c r="J32" s="1" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="K32" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L32" s="1">
         <v>2</v>
@@ -2290,10 +2350,10 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C33" s="3">
         <v>3</v>
@@ -2301,20 +2361,20 @@
       <c r="D33" s="3">
         <v>2.7</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="5" t="s">
         <v>53</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>73</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="K33" s="1">
         <v>2</v>
       </c>
       <c r="L33" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M33" s="1">
         <v>0</v>
@@ -2329,10 +2389,10 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="C34" s="3">
         <v>3</v>
@@ -2340,38 +2400,42 @@
       <c r="D34" s="3">
         <v>2.7</v>
       </c>
-      <c r="E34" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>80</v>
-      </c>
+      <c r="E34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="I34" s="11"/>
       <c r="J34" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="K34" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L34" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M34" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N34" s="1">
         <v>1</v>
       </c>
       <c r="O34" s="1">
         <f>K34*L34*M34*N34</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>56</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>64</v>
+        <v>39</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="C35" s="3">
         <v>3</v>
@@ -2380,37 +2444,37 @@
         <v>2.7</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>65</v>
+        <v>53</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="K35" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L35" s="1">
         <v>2</v>
       </c>
       <c r="M35" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N35" s="1">
         <v>1</v>
       </c>
       <c r="O35" s="1">
         <f>K35*L35*M35*N35</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>69</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>159</v>
+        <v>50</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="C36" s="3">
         <v>3</v>
@@ -2418,142 +2482,159 @@
       <c r="D36" s="3">
         <v>2.7</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>160</v>
+      <c r="E36" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>161</v>
+        <v>97</v>
+      </c>
+      <c r="K36" s="1">
+        <v>1</v>
+      </c>
+      <c r="L36" s="1">
+        <v>3</v>
+      </c>
+      <c r="M36" s="1">
+        <v>1</v>
+      </c>
+      <c r="N36" s="1">
+        <v>1</v>
+      </c>
+      <c r="O36" s="1">
+        <f>K36*L36*M36*N36</f>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>1</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E37" s="5"/>
+        <v>56</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" s="3">
+        <v>3</v>
+      </c>
+      <c r="D37" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>111</v>
+      </c>
       <c r="K37" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L37" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M37" s="1">
         <v>1</v>
       </c>
       <c r="N37" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O37" s="1">
         <f>K37*L37*M37*N37</f>
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>3</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E38" s="5"/>
-      <c r="K38" s="1">
-        <v>1</v>
-      </c>
-      <c r="L38" s="1">
-        <v>3</v>
-      </c>
-      <c r="M38" s="1">
-        <v>1</v>
-      </c>
-      <c r="N38" s="1">
-        <v>5</v>
-      </c>
-      <c r="O38" s="1">
-        <f>K38*L38*M38*N38</f>
-        <v>15</v>
+        <v>69</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C38" s="3">
+        <v>3</v>
+      </c>
+      <c r="D38" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E39" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="E39" s="5"/>
       <c r="K39" s="1">
         <v>2</v>
       </c>
       <c r="L39" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M39" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N39" s="1">
         <v>5</v>
       </c>
       <c r="O39" s="1">
         <f>K39*L39*M39*N39</f>
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E40" s="5"/>
-      <c r="F40" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="K40" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L40" s="1">
         <v>3</v>
       </c>
       <c r="M40" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N40" s="1">
         <v>5</v>
       </c>
       <c r="O40" s="1">
         <f>K40*L40*M40*N40</f>
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E41" s="2"/>
       <c r="K41" s="1">
@@ -2563,65 +2644,65 @@
         <v>2</v>
       </c>
       <c r="M41" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N41" s="1">
         <v>5</v>
       </c>
       <c r="O41" s="1">
         <f>K41*L41*M41*N41</f>
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E42" s="5"/>
+      <c r="F42" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="K42" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L42" s="1">
         <v>3</v>
       </c>
       <c r="M42" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N42" s="1">
         <v>5</v>
       </c>
       <c r="O42" s="1">
         <f>K42*L42*M42*N42</f>
-        <v>15</v>
+        <v>60</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E43" s="2"/>
-      <c r="J43" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="K43" s="1">
         <v>2</v>
       </c>
       <c r="L43" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M43" s="1">
         <v>1</v>
@@ -2631,84 +2712,87 @@
       </c>
       <c r="O43" s="1">
         <f>K43*L43*M43*N43</f>
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E44" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="E44" s="5"/>
       <c r="K44" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L44" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M44" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N44" s="1">
         <v>5</v>
       </c>
       <c r="O44" s="1">
         <f>K44*L44*M44*N44</f>
-        <v>40</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E45" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="J45" s="1" t="s">
+        <v>100</v>
+      </c>
       <c r="K45" s="1">
         <v>2</v>
       </c>
       <c r="L45" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M45" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N45" s="1">
         <v>5</v>
       </c>
       <c r="O45" s="1">
         <f>K45*L45*M45*N45</f>
-        <v>80</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E46" s="2"/>
       <c r="K46" s="1">
         <v>2</v>
       </c>
       <c r="L46" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M46" s="1">
         <v>2</v>
@@ -2718,58 +2802,58 @@
       </c>
       <c r="O46" s="1">
         <f>K46*L46*M46*N46</f>
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E47" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="E47" s="5"/>
       <c r="K47" s="1">
         <v>2</v>
       </c>
       <c r="L47" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M47" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N47" s="1">
         <v>5</v>
       </c>
       <c r="O47" s="1">
         <f>K47*L47*M47*N47</f>
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E48" s="2"/>
       <c r="K48" s="1">
         <v>2</v>
       </c>
       <c r="L48" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M48" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N48" s="1">
         <v>5</v>
@@ -2781,21 +2865,21 @@
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E49" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="E49" s="2"/>
       <c r="K49" s="1">
         <v>2</v>
       </c>
       <c r="L49" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M49" s="1">
         <v>1</v>
@@ -2805,19 +2889,19 @@
       </c>
       <c r="O49" s="1">
         <f>K49*L49*M49*N49</f>
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E50" s="2"/>
       <c r="K50" s="1">
@@ -2827,33 +2911,33 @@
         <v>2</v>
       </c>
       <c r="M50" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N50" s="1">
         <v>5</v>
       </c>
       <c r="O50" s="1">
         <f>K50*L50*M50*N50</f>
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E51" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="E51" s="5"/>
       <c r="K51" s="1">
         <v>2</v>
       </c>
       <c r="L51" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M51" s="1">
         <v>1</v>
@@ -2863,19 +2947,19 @@
       </c>
       <c r="O51" s="1">
         <f>K51*L51*M51*N51</f>
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E52" s="2"/>
       <c r="K52" s="1">
@@ -2885,33 +2969,33 @@
         <v>2</v>
       </c>
       <c r="M52" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N52" s="1">
         <v>5</v>
       </c>
       <c r="O52" s="1">
         <f>K52*L52*M52*N52</f>
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E53" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="E53" s="2"/>
       <c r="K53" s="1">
         <v>2</v>
       </c>
       <c r="L53" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M53" s="1">
         <v>1</v>
@@ -2921,26 +3005,26 @@
       </c>
       <c r="O53" s="1">
         <f>K53*L53*M53*N53</f>
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E54" s="2"/>
       <c r="K54" s="1">
         <v>2</v>
       </c>
       <c r="L54" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M54" s="1">
         <v>1</v>
@@ -2950,19 +3034,19 @@
       </c>
       <c r="O54" s="1">
         <f>K54*L54*M54*N54</f>
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E55" s="5"/>
       <c r="K55" s="1">
@@ -2984,19 +3068,16 @@
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>34</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C56" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56" s="3"/>
       <c r="D56" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E56" s="2"/>
-      <c r="J56" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="K56" s="1">
         <v>2</v>
       </c>
@@ -3007,148 +3088,147 @@
         <v>1</v>
       </c>
       <c r="N56" s="1">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="O56" s="1">
         <f>K56*L56*M56*N56</f>
-        <v>198</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>35</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C57" s="4"/>
+        <v>33</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C57" s="3"/>
       <c r="D57" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E57" s="2"/>
-      <c r="J57" s="1" t="s">
-        <v>118</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="E57" s="5"/>
       <c r="K57" s="1">
         <v>2</v>
       </c>
       <c r="L57" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M57" s="1">
         <v>1</v>
       </c>
       <c r="N57" s="1">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="O57" s="1">
         <f>K57*L57*M57*N57</f>
-        <v>198</v>
+        <v>30</v>
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>37</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C58" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C58" s="4"/>
       <c r="D58" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E58" s="2"/>
+      <c r="J58" s="1" t="s">
+        <v>114</v>
+      </c>
       <c r="K58" s="1">
         <v>2</v>
       </c>
       <c r="L58" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M58" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N58" s="1">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="O58" s="1">
         <f>K58*L58*M58*N58</f>
-        <v>40</v>
+        <v>198</v>
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>40</v>
-      </c>
-      <c r="B59" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C59" s="3"/>
+      <c r="B59" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59" s="4"/>
       <c r="D59" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E59" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="J59" s="1" t="s">
+        <v>115</v>
+      </c>
       <c r="K59" s="1">
         <v>2</v>
       </c>
       <c r="L59" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M59" s="1">
         <v>1</v>
       </c>
       <c r="N59" s="1">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="O59" s="1">
         <f>K59*L59*M59*N59</f>
-        <v>30</v>
+        <v>198</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E60" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="E60" s="2"/>
       <c r="K60" s="1">
         <v>2</v>
       </c>
       <c r="L60" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M60" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N60" s="1">
         <v>5</v>
       </c>
       <c r="O60" s="1">
         <f>K60*L60*M60*N60</f>
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E61" s="5"/>
-      <c r="H61" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="I61" s="10"/>
       <c r="K61" s="1">
         <v>2</v>
       </c>
@@ -3168,14 +3248,14 @@
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E62" s="5"/>
       <c r="K62" s="1">
@@ -3197,16 +3277,20 @@
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C63" s="3"/>
       <c r="D63" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E63" s="5"/>
+      <c r="H63" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="I63" s="10"/>
       <c r="K63" s="1">
         <v>2</v>
       </c>
@@ -3226,21 +3310,21 @@
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C64" s="3"/>
       <c r="D64" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E64" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="E64" s="5"/>
       <c r="K64" s="1">
         <v>2</v>
       </c>
       <c r="L64" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M64" s="1">
         <v>1</v>
@@ -3250,19 +3334,19 @@
       </c>
       <c r="O64" s="1">
         <f>K64*L64*M64*N64</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C65" s="3"/>
       <c r="D65" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E65" s="5"/>
       <c r="K65" s="1">
@@ -3284,21 +3368,21 @@
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C66" s="3"/>
       <c r="D66" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E66" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="E66" s="2"/>
       <c r="K66" s="1">
         <v>2</v>
       </c>
       <c r="L66" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M66" s="1">
         <v>1</v>
@@ -3308,59 +3392,52 @@
       </c>
       <c r="O66" s="1">
         <f>K66*L66*M66*N66</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A67" s="6">
-        <v>51</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C67" s="4"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>48</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C67" s="3"/>
       <c r="D67" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E67" s="7"/>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
-      <c r="H67" s="6"/>
-      <c r="I67" s="6"/>
-      <c r="J67" s="1" t="s">
-        <v>109</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="E67" s="5"/>
       <c r="K67" s="1">
         <v>2</v>
       </c>
-      <c r="L67" s="6">
-        <v>1</v>
-      </c>
-      <c r="M67" s="6">
-        <v>1</v>
-      </c>
-      <c r="N67" s="6">
-        <v>99</v>
+      <c r="L67" s="1">
+        <v>3</v>
+      </c>
+      <c r="M67" s="1">
+        <v>1</v>
+      </c>
+      <c r="N67" s="1">
+        <v>5</v>
       </c>
       <c r="O67" s="1">
         <f>K67*L67*M67*N67</f>
-        <v>198</v>
+        <v>30</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C68" s="3"/>
       <c r="D68" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E68" s="5"/>
       <c r="K68" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L68" s="1">
         <v>3</v>
@@ -3373,59 +3450,62 @@
       </c>
       <c r="O68" s="1">
         <f>K68*L68*M68*N68</f>
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A69" s="1">
-        <v>55</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>63</v>
-      </c>
+      <c r="A69" s="6">
+        <v>51</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C69" s="4"/>
       <c r="D69" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E69" s="2"/>
-      <c r="F69" s="1" t="s">
-        <v>66</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="E69" s="7"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="6"/>
       <c r="J69" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K69" s="1">
         <v>2</v>
       </c>
-      <c r="L69" s="1">
-        <v>1</v>
-      </c>
-      <c r="M69" s="1">
-        <v>1</v>
-      </c>
-      <c r="N69" s="1">
-        <v>5</v>
+      <c r="L69" s="6">
+        <v>1</v>
+      </c>
+      <c r="M69" s="6">
+        <v>1</v>
+      </c>
+      <c r="N69" s="6">
+        <v>99</v>
       </c>
       <c r="O69" s="1">
         <f>K69*L69*M69*N69</f>
-        <v>10</v>
+        <v>198</v>
       </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>59</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>72</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C70" s="3"/>
       <c r="D70" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E70" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="E70" s="5"/>
       <c r="K70" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L70" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M70" s="1">
         <v>1</v>
@@ -3435,12 +3515,74 @@
       </c>
       <c r="O70" s="1">
         <f>K70*L70*M70*N70</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>55</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E71" s="2"/>
+      <c r="F71" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="K71" s="1">
+        <v>2</v>
+      </c>
+      <c r="L71" s="1">
+        <v>1</v>
+      </c>
+      <c r="M71" s="1">
+        <v>1</v>
+      </c>
+      <c r="N71" s="1">
+        <v>5</v>
+      </c>
+      <c r="O71" s="1">
+        <f>K71*L71*M71*N71</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>59</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E72" s="2"/>
+      <c r="K72" s="1">
+        <v>2</v>
+      </c>
+      <c r="L72" s="1">
+        <v>2</v>
+      </c>
+      <c r="M72" s="1">
+        <v>1</v>
+      </c>
+      <c r="N72" s="1">
+        <v>5</v>
+      </c>
+      <c r="O72" s="1">
+        <f>K72*L72*M72*N72</f>
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T61" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O70">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O72">
       <sortCondition ref="C1:C61"/>
     </sortState>
   </autoFilter>
@@ -3458,15 +3600,15 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="H15" r:id="rId1" tooltip="otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" xr:uid="{DC8291FA-BBBC-4164-AFDF-A14D5C37779A}"/>
-    <hyperlink ref="H26" r:id="rId2" tooltip="otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" xr:uid="{DA695823-06F7-4C4D-A0BB-56A71E8AB3AA}"/>
-    <hyperlink ref="H61" r:id="rId3" tooltip="otcc2023.ND.007_BasicPhysicalIntent.zip" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.007_BasicPhysicalIntent.zip" xr:uid="{73726784-3406-4A32-9F90-250F1899557B}"/>
-    <hyperlink ref="H23" r:id="rId4" tooltip="otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" xr:uid="{B1E96811-E3AB-4B6A-9B71-389668390DD1}"/>
-    <hyperlink ref="H24" r:id="rId5" xr:uid="{39007AE4-376B-4AFF-B690-2B1FD75ED6B2}"/>
-    <hyperlink ref="H25" r:id="rId6" xr:uid="{B85E8F47-7893-459C-8DC1-8BC4AA02A23B}"/>
-    <hyperlink ref="H27" r:id="rId7" xr:uid="{E38CDBF1-9601-4855-8DFD-AE8A6A3AD6BE}"/>
-    <hyperlink ref="H32" r:id="rId8" xr:uid="{D578898C-48FA-4D82-82AF-E6661888BC34}"/>
-    <hyperlink ref="H2" r:id="rId9" xr:uid="{09D95B53-BA52-41E5-AAC0-0F3CBDC9FC82}"/>
+    <hyperlink ref="H18" r:id="rId1" tooltip="otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" xr:uid="{DC8291FA-BBBC-4164-AFDF-A14D5C37779A}"/>
+    <hyperlink ref="H28" r:id="rId2" tooltip="otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" xr:uid="{DA695823-06F7-4C4D-A0BB-56A71E8AB3AA}"/>
+    <hyperlink ref="H63" r:id="rId3" tooltip="otcc2023.ND.007_BasicPhysicalIntent.zip" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.007_BasicPhysicalIntent.zip" xr:uid="{73726784-3406-4A32-9F90-250F1899557B}"/>
+    <hyperlink ref="H17" r:id="rId4" tooltip="otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" xr:uid="{B1E96811-E3AB-4B6A-9B71-389668390DD1}"/>
+    <hyperlink ref="H26" r:id="rId5" xr:uid="{39007AE4-376B-4AFF-B690-2B1FD75ED6B2}"/>
+    <hyperlink ref="H27" r:id="rId6" xr:uid="{B85E8F47-7893-459C-8DC1-8BC4AA02A23B}"/>
+    <hyperlink ref="H29" r:id="rId7" xr:uid="{E38CDBF1-9601-4855-8DFD-AE8A6A3AD6BE}"/>
+    <hyperlink ref="H34" r:id="rId8" xr:uid="{D578898C-48FA-4D82-82AF-E6661888BC34}"/>
+    <hyperlink ref="H4" r:id="rId9" xr:uid="{09D95B53-BA52-41E5-AAC0-0F3CBDC9FC82}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Including operator priorities and analysis
</commit_message>
<xml_diff>
--- a/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
+++ b/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cienacorp-my.sharepoint.com/personal/ndavis_ciena_com/Documents/Documents/WorkingDocuments/BluePlanet/ApiPo/Standards/TAPI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7CCD126-8F49-4E8D-8D1F-2D2225682C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{769F7A87-A2C2-495B-A576-ECDB50264FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
+    <workbookView xWindow="-28875" yWindow="-16380" windowWidth="29040" windowHeight="16440" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$T$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$U$72</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="233">
   <si>
     <t>Feature</t>
   </si>
@@ -596,12 +596,196 @@
   <si>
     <t>#635</t>
   </si>
+  <si>
+    <t>Related docs</t>
+  </si>
+  <si>
+    <t>TIP MUST Priority</t>
+  </si>
+  <si>
+    <t>MUST 1,2,3</t>
+  </si>
+  <si>
+    <t>TIP MUST Comments</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>Operators' Priorities: (5: Low); (3: Medium); (1: Mandatory)</t>
+  </si>
+  <si>
+    <t>Roadmap item requiring more discussions</t>
+  </si>
+  <si>
+    <t>There is a work item buried under this that needs to be pulled out separately and moved to priority 1. The overal work item can be moved to priority 2</t>
+  </si>
+  <si>
+    <t>Path computation use cases are draft.
+Clarify definition of Path.</t>
+  </si>
+  <si>
+    <t>Key for operators to have full support of ZR/ZR+ pluggable E2E SDN management in a multi-vendor environment</t>
+  </si>
+  <si>
+    <t>BUT is dependent on IETF. May be part in 2.7 and part beyond.</t>
+  </si>
+  <si>
+    <t>How does TAPI relate to the pluggables.
+Assume that the optical controller has read access to the transponders.
+Need to show how a router with coherent transceivers is represented in TAPI and how the Orchestrator absorbs this.</t>
+  </si>
+  <si>
+    <t>This is underway</t>
+  </si>
+  <si>
+    <t>This is future</t>
+  </si>
+  <si>
+    <t>This is reasonable (but then the protobuf file should be backported).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Important to expose in a standard way in NBI some specific power measurement values at Add/Drop Rx/Tx? </t>
+  </si>
+  <si>
+    <t>Can add this. It is significant work, but achaievable.</t>
+  </si>
+  <si>
+    <t>What is really missing today in the T-API vs IETF? Perhaps Esther knows?</t>
+  </si>
+  <si>
+    <t>This is a validation task</t>
+  </si>
+  <si>
+    <t>interesting for future use cases</t>
+  </si>
+  <si>
+    <t>More a RIA consistency /cleaning regarding Mandatory/Optional/Condicional attributes</t>
+  </si>
+  <si>
+    <t>We can do this in background</t>
+  </si>
+  <si>
+    <t>scope unclear. No issues opened in Github</t>
+  </si>
+  <si>
+    <t>I suspect this will be elevated!</t>
+  </si>
+  <si>
+    <t>Difference in gNMI between on-change and sample</t>
+  </si>
+  <si>
+    <t>Could do this in background and prepare. Unlikely to be in 2.7.</t>
+  </si>
+  <si>
+    <t>Need to clarify this work.</t>
+  </si>
+  <si>
+    <t>As in TIP T-APIv2.1 TRD consolidating everything towards a single streaming strategy also for notifications</t>
+  </si>
+  <si>
+    <t>This is reasonable, but is significant work</t>
+  </si>
+  <si>
+    <t>Reverse should be true as well from T-API to IETF. Backward compatibility is key for operators with T-API</t>
+  </si>
+  <si>
+    <t>Related with the testing framework. Separate workstream</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>More a RIA update/cleaning issue</t>
+  </si>
+  <si>
+    <t>This is background</t>
+  </si>
+  <si>
+    <t>This is minor work and can be done</t>
+  </si>
+  <si>
+    <t>This is a fix to an incorrect approach.</t>
+  </si>
+  <si>
+    <t>Key for a standard implementation to expose LLDP key parameters (Chassis-ID, port-ID) intercepted by transponders/muxponders supporting LLDP snooping.</t>
+  </si>
+  <si>
+    <t>Improvement for UC 0d (multi-domain OTN interdomain links discovery using OTN TTI. For supporting more G709 fields then just SAPI/DAPI which have a length limitation. Eg. Operator field could be supported to remove that limitation</t>
+  </si>
+  <si>
+    <t>More a RIA update issue</t>
+  </si>
+  <si>
+    <t>Remove unnecessary string restrictions in INVENTORY_ID for use cases 4a/4b</t>
+  </si>
+  <si>
+    <t>Not required by VF but understand other TIP operators would like to have it in T-APIv2.1.4.</t>
+  </si>
+  <si>
+    <t>This is a T-APIV2.5 fix to allow the use of protobuf file for applying fixes as it is done in T-APIv2.6</t>
+  </si>
+  <si>
+    <t>We need this to operate. It is not a feature.</t>
+  </si>
+  <si>
+    <t>Same as above and done now in T-APIv2.5 as in T-APIv2.6</t>
+  </si>
+  <si>
+    <t>This is straight forward and has major benefits</t>
+  </si>
+  <si>
+    <t>See presentation from Nigel Davis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Different behaviours between Vendors in their implementations regarding service/connection LCM. Important to be fixed for higher interoperability </t>
+  </si>
+  <si>
+    <t>Needs significant work</t>
+  </si>
+  <si>
+    <t>Key to align between all organisations to allow E2E SDN management of ZR(+) pluggables in the router over OLS in a multi-vendor environment</t>
+  </si>
+  <si>
+    <t>This is a coordination activity. There is an initiative in OIF that we could join with formally.</t>
+  </si>
+  <si>
+    <t>Application descriptors etc. 
+Proprietary properties</t>
+  </si>
+  <si>
+    <t>ND/RC</t>
+  </si>
+  <si>
+    <t>#637</t>
+  </si>
+  <si>
+    <t>#638</t>
+  </si>
+  <si>
+    <t>#639</t>
+  </si>
+  <si>
+    <t>#640</t>
+  </si>
+  <si>
+    <t>#641</t>
+  </si>
+  <si>
+    <t>#643</t>
+  </si>
+  <si>
+    <t>#642</t>
+  </si>
+  <si>
+    <t>#644</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -657,8 +841,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -689,8 +896,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFAFAF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF99FF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -698,12 +929,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -750,12 +1009,62 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF99FF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFAFAF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1090,28 +1399,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O72"/>
+  <dimension ref="A1:U72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="71" style="1" customWidth="1"/>
+    <col min="2" max="2" width="63.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="6.42578125" style="1" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="9.140625" style="1"/>
     <col min="7" max="7" width="23.5703125" style="1" customWidth="1"/>
     <col min="8" max="8" width="51.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="29.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="81.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="40.85546875" style="1" customWidth="1"/>
     <col min="11" max="11" width="9.140625" style="1" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="12.85546875" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="15.140625" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="18" style="1" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="10.85546875" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="1"/>
+    <col min="16" max="17" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.42578125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="14.5703125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="31" style="1" customWidth="1"/>
+    <col min="21" max="21" width="20.140625" style="1" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
@@ -1133,6 +1447,9 @@
       <c r="G1" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>173</v>
+      </c>
       <c r="I1" s="1" t="s">
         <v>144</v>
       </c>
@@ -1154,129 +1471,216 @@
       <c r="O1" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="P1" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q1" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="R1" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="U1" s="17" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>70</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="C2" s="15">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>107</v>
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>159</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="I2" s="14" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="I2" s="10"/>
+      <c r="J2" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="K2" s="1">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1">
+        <v>3</v>
+      </c>
+      <c r="M2" s="1">
+        <v>1</v>
+      </c>
+      <c r="N2" s="1">
+        <v>1</v>
+      </c>
+      <c r="O2" s="1">
+        <f>K2*L2*M2*N2</f>
+        <v>3</v>
+      </c>
+      <c r="P2" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="18">
+        <v>1</v>
+      </c>
+      <c r="R2" s="18"/>
+      <c r="S2" s="1" t="str">
+        <f>IF(Q2="", "?",IF(Q2="?", "?", IF(C2=Q2, "-",IF(C2&gt;Q2,"H",IF(C2&lt;Q2,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T2" s="21"/>
+    </row>
+    <row r="3" spans="1:21" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C3" s="15">
-        <v>0</v>
+        <v>67</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1</v>
       </c>
       <c r="D3" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>107</v>
+        <v>2.7</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K3" s="1">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1">
+        <v>2</v>
+      </c>
+      <c r="M3" s="1">
+        <v>1</v>
+      </c>
+      <c r="N3" s="1">
+        <v>1</v>
+      </c>
+      <c r="O3" s="1">
+        <f>K3*L3*M3*N3</f>
+        <v>2</v>
+      </c>
+      <c r="P3" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="18">
+        <v>1</v>
+      </c>
+      <c r="R3" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="S3" s="1" t="str">
+        <f>IF(Q3="", "?",IF(Q3="?", "?", IF(C3=Q3, "-",IF(C3&gt;Q3,"H",IF(C3&lt;Q3,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T3" s="21"/>
+    </row>
+    <row r="4" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>15</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>62</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="C4" s="3">
         <v>1</v>
       </c>
-      <c r="D4" s="3">
-        <v>2.7</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>159</v>
+      <c r="D4" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="I4" s="10"/>
-      <c r="J4" s="1" t="s">
-        <v>161</v>
+        <v>129</v>
       </c>
       <c r="K4" s="1">
         <v>1</v>
       </c>
       <c r="L4" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" s="1">
         <v>1</v>
       </c>
       <c r="O4" s="1">
         <f>K4*L4*M4*N4</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="P4" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="18">
+        <v>1</v>
+      </c>
+      <c r="R4" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="S4" s="1" t="str">
+        <f>IF(Q4="", "?",IF(Q4="?", "?", IF(C4=Q4, "-",IF(C4&gt;Q4,"H",IF(C4&lt;Q4,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T4" s="21"/>
+    </row>
+    <row r="5" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>18</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>63</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="C5" s="3">
         <v>1</v>
       </c>
-      <c r="D5" s="3">
-        <v>2.7</v>
+      <c r="D5" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>84</v>
+        <v>153</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="K5" s="1">
         <v>1</v>
       </c>
       <c r="L5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" s="1">
         <v>1</v>
@@ -1286,36 +1690,47 @@
       </c>
       <c r="O5" s="1">
         <f>K5*L5*M5*N5</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="P5" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="18">
+        <v>1</v>
+      </c>
+      <c r="R5" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="S5" s="1" t="str">
+        <f>IF(Q5="", "?",IF(Q5="?", "?", IF(C5=Q5, "-",IF(C5&gt;Q5,"H",IF(C5&lt;Q5,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T5" s="21"/>
+    </row>
+    <row r="6" spans="1:21" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>61</v>
+        <v>148</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>132</v>
+      <c r="D6" s="3">
+        <v>2.7</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>89</v>
+        <v>149</v>
       </c>
       <c r="K6" s="1">
         <v>1</v>
       </c>
       <c r="L6" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" s="1">
         <v>1</v>
@@ -1325,15 +1740,29 @@
       </c>
       <c r="O6" s="1">
         <f>K6*L6*M6*N6</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="P6" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="18">
+        <v>1</v>
+      </c>
+      <c r="R6" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="S6" s="1" t="str">
+        <f>IF(Q6="", "?",IF(Q6="?", "?", IF(C6=Q6, "-",IF(C6&gt;Q6,"H",IF(C6&lt;Q6,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T6" s="21"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
@@ -1342,58 +1771,60 @@
         <v>2.7</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>105</v>
+        <v>150</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="K7" s="1">
-        <v>1</v>
-      </c>
-      <c r="L7" s="1">
-        <v>2</v>
-      </c>
-      <c r="M7" s="1">
-        <v>1</v>
-      </c>
-      <c r="N7" s="1">
-        <v>1</v>
-      </c>
-      <c r="O7" s="1">
-        <f>K7*L7*M7*N7</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+      <c r="P7" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="18">
+        <v>1</v>
+      </c>
+      <c r="R7" s="18"/>
+      <c r="S7" s="1" t="str">
+        <f>IF(Q7="", "?",IF(Q7="?", "?", IF(C7=Q7, "-",IF(C7&gt;Q7,"H",IF(C7&lt;Q7,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>58</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="C8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="3">
         <v>2.7</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>70</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="I8" s="10"/>
       <c r="J8" s="1" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="K8" s="1">
         <v>1</v>
       </c>
       <c r="L8" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="1">
         <v>1</v>
@@ -1403,36 +1834,56 @@
       </c>
       <c r="O8" s="1">
         <f>K8*L8*M8*N8</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="P8" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="18">
+        <v>1</v>
+      </c>
+      <c r="R8" s="18"/>
+      <c r="S8" s="1" t="str">
+        <f>IF(Q8="", "?",IF(Q8="?", "?", IF(C8=Q8, "-",IF(C8&gt;Q8,"H",IF(C8&lt;Q8,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T8" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>61</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>127</v>
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="C9" s="3">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>132</v>
+        <v>2</v>
+      </c>
+      <c r="D9" s="3">
+        <v>2.7</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>128</v>
+        <v>171</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="K9" s="1">
         <v>1</v>
       </c>
       <c r="L9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="1">
         <v>1</v>
@@ -1441,73 +1892,112 @@
         <f>K9*L9*M9*N9</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="P9" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="18">
+        <v>1</v>
+      </c>
+      <c r="R9" s="18"/>
+      <c r="S9" s="1" t="str">
+        <f>IF(Q9="", "?",IF(Q9="?", "?", IF(C9=Q9, "-",IF(C9&gt;Q9,"H",IF(C9&lt;Q9,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T9" s="21" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>62</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>134</v>
+        <v>30</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>74</v>
       </c>
       <c r="C10" s="3">
-        <v>1</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>53</v>
+        <v>2</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>86</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>129</v>
+        <v>172</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
       </c>
       <c r="L10" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M10" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N10" s="1">
         <v>1</v>
       </c>
       <c r="O10" s="1">
         <f>K10*L10*M10*N10</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="P10" s="22">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="22">
+        <v>1</v>
+      </c>
+      <c r="R10" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="S10" s="1" t="str">
+        <f>IF(Q10="", "?",IF(Q10="?", "?", IF(C10=Q10, "-",IF(C10&gt;Q10,"H",IF(C10&lt;Q10,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="U10" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>63</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>135</v>
+        <v>31</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="C11" s="3">
-        <v>1</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>53</v>
+        <v>2</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>86</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>136</v>
+        <v>60</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>90</v>
       </c>
       <c r="K11" s="1">
         <v>1</v>
       </c>
       <c r="L11" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M11" s="1">
         <v>1</v>
@@ -1517,27 +2007,53 @@
       </c>
       <c r="O11" s="1">
         <f>K11*L11*M11*N11</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="P11" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="18">
+        <v>1</v>
+      </c>
+      <c r="R11" s="18" t="s">
+        <v>200</v>
+      </c>
+      <c r="S11" s="1" t="str">
+        <f>IF(Q11="", "?",IF(Q11="?", "?", IF(C11=Q11, "-",IF(C11&gt;Q11,"H",IF(C11&lt;Q11,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T11" s="21" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" ht="225" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>64</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>137</v>
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>5</v>
       </c>
       <c r="C12" s="3">
-        <v>1</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>139</v>
+        <v>3</v>
+      </c>
+      <c r="D12" s="3">
+        <v>2.7</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>53</v>
+        <v>224</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>138</v>
+        <v>225</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="I12" s="11"/>
+      <c r="J12" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="K12" s="1">
         <v>1</v>
@@ -1546,40 +2062,69 @@
         <v>2</v>
       </c>
       <c r="M12" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N12" s="1">
         <v>1</v>
       </c>
       <c r="O12" s="1">
         <f>K12*L12*M12*N12</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="P12" s="20">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="20">
+        <v>1</v>
+      </c>
+      <c r="R12" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="S12" s="1" t="str">
+        <f>IF(Q12="", "?",IF(Q12="?", "?", IF(C12=Q12, "-",IF(C12&gt;Q12,"H",IF(C12&lt;Q12,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T12" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>65</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>140</v>
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="C13" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="E13" s="2" t="s">
+        <v>2.7</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>53</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>141</v>
+        <v>226</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="I13" s="10"/>
+      <c r="J13" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="K13" s="1">
         <v>1</v>
       </c>
       <c r="L13" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M13" s="1">
         <v>1</v>
@@ -1589,54 +2134,74 @@
       </c>
       <c r="O13" s="1">
         <f>K13*L13*M13*N13</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="P13" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="18">
+        <v>1</v>
+      </c>
+      <c r="R13" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="S13" s="1" t="str">
+        <f>IF(Q13="", "?",IF(Q13="?", "?", IF(C13=Q13, "-",IF(C13&gt;Q13,"H",IF(C13&lt;Q13,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T13" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="U13" s="6"/>
+    </row>
+    <row r="14" spans="1:21" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="C14" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="3">
         <v>2.7</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>53</v>
+        <v>156</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="K14" s="1">
-        <v>1</v>
-      </c>
-      <c r="L14" s="1">
-        <v>1</v>
-      </c>
-      <c r="M14" s="1">
-        <v>1</v>
-      </c>
-      <c r="N14" s="1">
-        <v>1</v>
-      </c>
-      <c r="O14" s="1">
-        <f>K14*L14*M14*N14</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P14" s="20">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="20">
+        <v>1</v>
+      </c>
+      <c r="R14" s="24" t="s">
+        <v>221</v>
+      </c>
+      <c r="S14" s="1" t="str">
+        <f>IF(Q14="", "?",IF(Q14="?", "?", IF(C14=Q14, "-",IF(C14&gt;Q14,"H",IF(C14&lt;Q14,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T14" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>148</v>
+        <v>69</v>
       </c>
       <c r="C15" s="3">
         <v>1</v>
@@ -1645,16 +2210,19 @@
         <v>2.7</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>149</v>
+        <v>70</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="K15" s="1">
         <v>1</v>
       </c>
       <c r="L15" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M15" s="1">
         <v>1</v>
@@ -1664,63 +2232,104 @@
       </c>
       <c r="O15" s="1">
         <f>K15*L15*M15*N15</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="P15" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q15" s="18">
+        <v>2</v>
+      </c>
+      <c r="R15" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="S15" s="1" t="str">
+        <f>IF(Q15="", "?",IF(Q15="?", "?", IF(C15=Q15, "-",IF(C15&gt;Q15,"H",IF(C15&lt;Q15,"L")))))</f>
+        <v>L</v>
+      </c>
+      <c r="T15" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>47</v>
+        <v>137</v>
       </c>
       <c r="C16" s="3">
         <v>1</v>
       </c>
-      <c r="D16" s="3">
-        <v>2.7</v>
+      <c r="D16" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>150</v>
+        <v>53</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+      <c r="K16" s="1">
+        <v>1</v>
+      </c>
+      <c r="L16" s="1">
+        <v>2</v>
+      </c>
+      <c r="M16" s="1">
+        <v>2</v>
+      </c>
+      <c r="N16" s="1">
+        <v>1</v>
+      </c>
+      <c r="O16" s="1">
+        <f>K16*L16*M16*N16</f>
+        <v>4</v>
+      </c>
+      <c r="P16" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="18">
+        <v>2</v>
+      </c>
+      <c r="R16" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="S16" s="1" t="str">
+        <f>IF(Q16="", "?",IF(Q16="?", "?", IF(C16=Q16, "-",IF(C16&gt;Q16,"H",IF(C16&lt;Q16,"L")))))</f>
+        <v>L</v>
+      </c>
+      <c r="T16" s="23" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>2</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C17" s="13">
-        <v>2</v>
+        <v>66</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C17" s="3">
+        <v>1</v>
       </c>
       <c r="D17" s="3">
         <v>2.7</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="I17" s="10"/>
-      <c r="J17" s="1" t="s">
-        <v>160</v>
+      <c r="F17" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="K17" s="1">
         <v>1</v>
       </c>
       <c r="L17" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M17" s="1">
         <v>1</v>
@@ -1730,43 +2339,59 @@
       </c>
       <c r="O17" s="1">
         <f>K17*L17*M17*N17</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="P17" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q17" s="18">
+        <v>2</v>
+      </c>
+      <c r="R17" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="S17" s="1" t="str">
+        <f>IF(Q17="", "?",IF(Q17="?", "?", IF(C17=Q17, "-",IF(C17&gt;Q17,"H",IF(C17&lt;Q17,"L")))))</f>
+        <v>L</v>
+      </c>
+      <c r="T17" s="23" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="3">
+        <v>2</v>
+      </c>
+      <c r="C18" s="13">
         <v>2</v>
       </c>
       <c r="D18" s="3">
         <v>2.7</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>170</v>
+      <c r="F18" s="12" t="s">
+        <v>158</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I18" s="10"/>
       <c r="J18" s="1" t="s">
-        <v>88</v>
+        <v>160</v>
       </c>
       <c r="K18" s="1">
         <v>1</v>
       </c>
       <c r="L18" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M18" s="1">
         <v>1</v>
@@ -1776,15 +2401,34 @@
       </c>
       <c r="O18" s="1">
         <f>K18*L18*M18*N18</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="P18" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q18" s="18">
+        <v>2</v>
+      </c>
+      <c r="R18" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="S18" s="1" t="str">
+        <f>IF(Q18="", "?",IF(Q18="?", "?", IF(C18=Q18, "-",IF(C18&gt;Q18,"H",IF(C18&lt;Q18,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T18" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>9</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>7</v>
+        <v>53</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>58</v>
       </c>
       <c r="C19" s="3">
         <v>2</v>
@@ -1793,25 +2437,19 @@
         <v>2.7</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="K19" s="1">
         <v>1</v>
       </c>
       <c r="L19" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M19" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N19" s="1">
         <v>1</v>
@@ -1820,124 +2458,176 @@
         <f>K19*L19*M19*N19</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="P19" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q19" s="18">
+        <v>2</v>
+      </c>
+      <c r="R19" s="18"/>
+      <c r="S19" s="1" t="str">
+        <f>IF(Q19="", "?",IF(Q19="?", "?", IF(C19=Q19, "-",IF(C19&gt;Q19,"H",IF(C19&lt;Q19,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="C20" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" s="3">
         <v>2.7</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>86</v>
+      <c r="E20" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>80</v>
-      </c>
+        <v>228</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="I20" s="11"/>
       <c r="J20" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="K20" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L20" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M20" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N20" s="1">
         <v>1</v>
       </c>
       <c r="O20" s="1">
         <f>K20*L20*M20*N20</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="P20" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q20" s="18">
+        <v>2</v>
+      </c>
+      <c r="R20" s="18"/>
+      <c r="S20" s="1" t="str">
+        <f>IF(Q20="", "?",IF(Q20="?", "?", IF(C20=Q20, "-",IF(C20&gt;Q20,"H",IF(C20&lt;Q20,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T20" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C21" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="3">
         <v>2.7</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>86</v>
+      <c r="E21" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>90</v>
+        <v>229</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="I21" s="11"/>
+      <c r="J21" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="K21" s="1">
         <v>1</v>
       </c>
       <c r="L21" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M21" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N21" s="1">
         <v>1</v>
       </c>
       <c r="O21" s="1">
         <f>K21*L21*M21*N21</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="P21" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q21" s="18">
+        <v>2</v>
+      </c>
+      <c r="R21" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="S21" s="1" t="str">
+        <f>IF(Q21="", "?",IF(Q21="?", "?", IF(C21=Q21, "-",IF(C21&gt;Q21,"H",IF(C21&lt;Q21,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T21" s="21" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C22" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D22" s="3">
         <v>2.7</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>152</v>
+        <v>231</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K22" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22" s="1">
         <v>2</v>
       </c>
       <c r="M22" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N22" s="1">
         <v>1</v>
@@ -1946,16 +2636,32 @@
         <f>K22*L22*M22*N22</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="P22" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q22" s="18">
+        <v>2</v>
+      </c>
+      <c r="R22" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="S22" s="1" t="str">
+        <f>IF(Q22="", "?",IF(Q22="?", "?", IF(C22=Q22, "-",IF(C22&gt;Q22,"H",IF(C22&lt;Q22,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T22" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C23" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" s="3">
         <v>2.7</v>
@@ -1963,96 +2669,140 @@
       <c r="E23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I23" s="12" t="s">
-        <v>169</v>
-      </c>
+      <c r="F23" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="I23" s="11"/>
       <c r="J23" s="1" t="s">
-        <v>168</v>
+        <v>93</v>
       </c>
       <c r="K23" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L23" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M23" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" s="1">
         <v>1</v>
       </c>
       <c r="O23" s="1">
         <f>K23*L23*M23*N23</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="P23" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q23" s="18">
+        <v>2</v>
+      </c>
+      <c r="R23" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="S23" s="1" t="str">
+        <f>IF(Q23="", "?",IF(Q23="?", "?", IF(C23=Q23, "-",IF(C23&gt;Q23,"H",IF(C23&lt;Q23,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T23" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>53</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>58</v>
+        <v>39</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="C24" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D24" s="3">
         <v>2.7</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>107</v>
+        <v>53</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G24" s="1"/>
+        <v>232</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>73</v>
+      </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
+      <c r="J24" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="K24" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L24" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M24" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N24" s="1">
         <v>1</v>
       </c>
       <c r="O24" s="1">
         <f>K24*L24*M24*N24</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="P24" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q24" s="18">
+        <v>2</v>
+      </c>
+      <c r="R24" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="S24" s="1" t="str">
+        <f>IF(Q24="", "?",IF(Q24="?", "?", IF(C24=Q24, "-",IF(C24&gt;Q24,"H",IF(C24&lt;Q24,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T24" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="U24" s="1"/>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>108</v>
+        <v>64</v>
       </c>
       <c r="C25" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" s="3">
         <v>2.7</v>
       </c>
-      <c r="E25" s="5" t="s">
-        <v>53</v>
+      <c r="E25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>65</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K25" s="1">
         <v>1</v>
       </c>
       <c r="L25" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M25" s="1">
         <v>1</v>
@@ -2062,18 +2812,32 @@
       </c>
       <c r="O25" s="1">
         <f>K25*L25*M25*N25</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="P25" s="18">
+        <v>3</v>
+      </c>
+      <c r="Q25" s="18">
+        <v>2</v>
+      </c>
+      <c r="R25" s="18"/>
+      <c r="S25" s="1" t="str">
+        <f>IF(Q25="", "?",IF(Q25="?", "?", IF(C25=Q25, "-",IF(C25&gt;Q25,"H",IF(C25&lt;Q25,"L")))))</f>
+        <v>H</v>
+      </c>
+      <c r="T25" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C26" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D26" s="3">
         <v>2.7</v>
@@ -2081,15 +2845,14 @@
       <c r="E26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H26" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="I26" s="11"/>
-      <c r="J26" s="1" t="s">
-        <v>91</v>
+      <c r="F26" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>84</v>
       </c>
       <c r="K26" s="1">
         <v>1</v>
@@ -2098,151 +2861,197 @@
         <v>2</v>
       </c>
       <c r="M26" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N26" s="1">
         <v>1</v>
       </c>
       <c r="O26" s="1">
         <f>K26*L26*M26*N26</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="P26" s="18">
+        <v>5</v>
+      </c>
+      <c r="Q26" s="18">
+        <v>3</v>
+      </c>
+      <c r="R26" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="S26" s="1" t="str">
+        <f>IF(Q26="", "?",IF(Q26="?", "?", IF(C26=Q26, "-",IF(C26&gt;Q26,"H",IF(C26&lt;Q26,"L")))))</f>
+        <v>L</v>
+      </c>
+      <c r="T26" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>8</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>123</v>
+        <v>54</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="C27" s="3">
-        <v>3</v>
-      </c>
-      <c r="D27" s="3">
-        <v>2.7</v>
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>132</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G27" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H27" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="I27" s="11"/>
+      <c r="F27" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="J27" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K27" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L27" s="1">
         <v>2</v>
       </c>
       <c r="M27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N27" s="1">
         <v>1</v>
       </c>
       <c r="O27" s="1">
         <f>K27*L27*M27*N27</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="P27" s="18">
+        <v>5</v>
+      </c>
+      <c r="Q27" s="18">
+        <v>3</v>
+      </c>
+      <c r="R27" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="S27" s="1" t="str">
+        <f>IF(Q27="", "?",IF(Q27="?", "?", IF(C27=Q27, "-",IF(C27&gt;Q27,"H",IF(C27&lt;Q27,"L")))))</f>
+        <v>L</v>
+      </c>
+      <c r="T27" s="23" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>10</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>8</v>
+        <v>61</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="C28" s="3">
-        <v>3</v>
-      </c>
-      <c r="D28" s="3">
-        <v>2.7</v>
-      </c>
-      <c r="E28" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H28" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="I28" s="10"/>
-      <c r="J28" s="1" t="s">
-        <v>95</v>
+      <c r="F28" s="1" t="s">
+        <v>128</v>
       </c>
       <c r="K28" s="1">
         <v>1</v>
       </c>
       <c r="L28" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M28" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N28" s="1">
         <v>1</v>
       </c>
       <c r="O28" s="1">
         <f>K28*L28*M28*N28</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="P28" s="18">
+        <v>5</v>
+      </c>
+      <c r="Q28" s="18">
+        <v>3</v>
+      </c>
+      <c r="R28" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="S28" s="1" t="str">
+        <f>IF(Q28="", "?",IF(Q28="?", "?", IF(C28=Q28, "-",IF(C28&gt;Q28,"H",IF(C28&lt;Q28,"L")))))</f>
+        <v>L</v>
+      </c>
+      <c r="T28" s="23" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>12</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>10</v>
+        <v>65</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C29" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D29" s="3">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H29" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="I29" s="11"/>
-      <c r="J29" s="1" t="s">
-        <v>91</v>
+      <c r="F29" s="1" t="s">
+        <v>141</v>
       </c>
       <c r="K29" s="1">
         <v>1</v>
       </c>
       <c r="L29" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M29" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N29" s="1">
         <v>1</v>
       </c>
       <c r="O29" s="1">
         <f>K29*L29*M29*N29</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="P29" s="18">
+        <v>5</v>
+      </c>
+      <c r="Q29" s="18">
+        <v>3</v>
+      </c>
+      <c r="R29" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="S29" s="1" t="str">
+        <f>IF(Q29="", "?",IF(Q29="?", "?", IF(C29=Q29, "-",IF(C29&gt;Q29,"H",IF(C29&lt;Q29,"L")))))</f>
+        <v>L</v>
+      </c>
+      <c r="T29" s="23" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>11</v>
+        <v>75</v>
       </c>
       <c r="C30" s="3">
         <v>3</v>
@@ -2253,35 +3062,49 @@
       <c r="E30" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G30" s="1" t="s">
-        <v>104</v>
+      <c r="G30" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="K30" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L30" s="1">
         <v>2</v>
       </c>
       <c r="M30" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N30" s="1">
         <v>1</v>
       </c>
       <c r="O30" s="1">
         <f>K30*L30*M30*N30</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="P30" s="18">
+        <v>5</v>
+      </c>
+      <c r="Q30" s="18">
+        <v>3</v>
+      </c>
+      <c r="R30" s="18"/>
+      <c r="S30" s="1" t="str">
+        <f>IF(Q30="", "?",IF(Q30="?", "?", IF(C30=Q30, "-",IF(C30&gt;Q30,"H",IF(C30&lt;Q30,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T30" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C31" s="3">
         <v>3</v>
@@ -2290,31 +3113,51 @@
         <v>2.7</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>109</v>
       </c>
       <c r="K31" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L31" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M31" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N31" s="1">
         <v>1</v>
       </c>
       <c r="O31" s="1">
         <f>K31*L31*M31*N31</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="P31" s="18">
+        <v>5</v>
+      </c>
+      <c r="Q31" s="18">
+        <v>3</v>
+      </c>
+      <c r="R31" s="18"/>
+      <c r="S31" s="1" t="str">
+        <f>IF(Q31="", "?",IF(Q31="?", "?", IF(C31=Q31, "-",IF(C31&gt;Q31,"H",IF(C31&lt;Q31,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T31" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="C32" s="3">
         <v>3</v>
@@ -2322,77 +3165,110 @@
       <c r="D32" s="3">
         <v>2.7</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>73</v>
+      <c r="E32" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="K32" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L32" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M32" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N32" s="1">
         <v>1</v>
       </c>
       <c r="O32" s="1">
         <f>K32*L32*M32*N32</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="P32" s="18">
+        <v>5</v>
+      </c>
+      <c r="Q32" s="18">
+        <v>3</v>
+      </c>
+      <c r="R32" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="S32" s="1" t="str">
+        <f>IF(Q32="", "?",IF(Q32="?", "?", IF(C32=Q32, "-",IF(C32&gt;Q32,"H",IF(C32&lt;Q32,"L")))))</f>
+        <v>-</v>
+      </c>
+      <c r="T32" s="21" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C33" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D33" s="3">
         <v>2.7</v>
       </c>
-      <c r="E33" s="5" t="s">
+      <c r="E33" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G33" s="2" t="s">
-        <v>73</v>
+      <c r="G33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>169</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="K33" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L33" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M33" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" s="1">
         <v>1</v>
       </c>
       <c r="O33" s="1">
         <f>K33*L33*M33*N33</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="P33" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q33" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="R33" s="22"/>
+      <c r="S33" s="1" t="str">
+        <f>IF(Q33="", "?",IF(Q33="?", "?", IF(C33=Q33, "-",IF(C33&gt;Q33,"H",IF(C33&lt;Q33,"L")))))</f>
+        <v>?</v>
+      </c>
+      <c r="T33" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="C34" s="3">
         <v>3</v>
@@ -2400,135 +3276,126 @@
       <c r="D34" s="3">
         <v>2.7</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H34" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="I34" s="11"/>
-      <c r="J34" s="1" t="s">
-        <v>93</v>
+      <c r="E34" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="K34" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L34" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M34" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N34" s="1">
         <v>1</v>
       </c>
       <c r="O34" s="1">
         <f>K34*L34*M34*N34</f>
+        <v>3</v>
+      </c>
+      <c r="P34" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q34" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="R34" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="S34" s="1" t="str">
+        <f>IF(Q34="", "?",IF(Q34="?", "?", IF(C34=Q34, "-",IF(C34&gt;Q34,"H",IF(C34&lt;Q34,"L")))))</f>
+        <v>?</v>
+      </c>
+      <c r="T34" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>70</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C35" s="15">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>39</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C35" s="3">
-        <v>3</v>
-      </c>
-      <c r="D35" s="3">
-        <v>2.7</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K35" s="1">
-        <v>2</v>
-      </c>
-      <c r="L35" s="1">
-        <v>2</v>
-      </c>
-      <c r="M35" s="1">
+      <c r="D35" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I35" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="P35" s="18"/>
+      <c r="Q35" s="18"/>
+      <c r="R35" s="18"/>
+      <c r="S35" s="1" t="str">
+        <f>IF(Q35="", "?",IF(Q35="?", "?", IF(C35=Q35, "-",IF(C35&gt;Q35,"H",IF(C35&lt;Q35,"L")))))</f>
+        <v>?</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>71</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C36" s="15">
         <v>0</v>
       </c>
-      <c r="N35" s="1">
-        <v>1</v>
-      </c>
-      <c r="O35" s="1">
-        <f>K35*L35*M35*N35</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>50</v>
-      </c>
-      <c r="B36" s="3" t="s">
+      <c r="D36" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="P36" s="18"/>
+      <c r="Q36" s="18"/>
+      <c r="R36" s="18"/>
+      <c r="S36" s="1" t="str">
+        <f>IF(Q36="", "?",IF(Q36="?", "?", IF(C36=Q36, "-",IF(C36&gt;Q36,"H",IF(C36&lt;Q36,"L")))))</f>
+        <v>?</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
         <v>45</v>
       </c>
-      <c r="C36" s="3">
-        <v>3</v>
-      </c>
-      <c r="D36" s="3">
-        <v>2.7</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K36" s="1">
-        <v>1</v>
-      </c>
-      <c r="L36" s="1">
-        <v>3</v>
-      </c>
-      <c r="M36" s="1">
-        <v>1</v>
-      </c>
-      <c r="N36" s="1">
-        <v>1</v>
-      </c>
-      <c r="O36" s="1">
-        <f>K36*L36*M36*N36</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <v>56</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>64</v>
+      <c r="B37" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="C37" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D37" s="3">
         <v>2.7</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>65</v>
+        <v>152</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="K37" s="1">
         <v>1</v>
@@ -2537,37 +3404,77 @@
         <v>2</v>
       </c>
       <c r="M37" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" s="1">
         <v>1</v>
       </c>
       <c r="O37" s="1">
         <f>K37*L37*M37*N37</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="P37" s="22"/>
+      <c r="Q37" s="22"/>
+      <c r="R37" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="S37" s="1" t="str">
+        <f>IF(Q37="", "?",IF(Q37="?", "?", IF(C37=Q37, "-",IF(C37&gt;Q37,"H",IF(C37&lt;Q37,"L")))))</f>
+        <v>?</v>
+      </c>
+      <c r="T37" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>155</v>
+        <v>108</v>
       </c>
       <c r="C38" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D38" s="3">
         <v>2.7</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>156</v>
+      <c r="E38" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="K38" s="1">
+        <v>1</v>
+      </c>
+      <c r="L38" s="1">
+        <v>3</v>
+      </c>
+      <c r="M38" s="1">
+        <v>1</v>
+      </c>
+      <c r="N38" s="1">
+        <v>1</v>
+      </c>
+      <c r="O38" s="1">
+        <f>K38*L38*M38*N38</f>
+        <v>3</v>
+      </c>
+      <c r="P38" s="22"/>
+      <c r="Q38" s="22"/>
+      <c r="R38" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="S38" s="1" t="str">
+        <f>IF(Q38="", "?",IF(Q38="?", "?", IF(C38=Q38, "-",IF(C38&gt;Q38,"H",IF(C38&lt;Q38,"L")))))</f>
+        <v>?</v>
+      </c>
+      <c r="T38" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>1</v>
       </c>
@@ -2595,8 +3502,11 @@
         <f>K39*L39*M39*N39</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P39" s="18"/>
+      <c r="Q39" s="18"/>
+      <c r="R39" s="18"/>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>3</v>
       </c>
@@ -2624,8 +3534,11 @@
         <f>K40*L40*M40*N40</f>
         <v>15</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P40" s="18"/>
+      <c r="Q40" s="18"/>
+      <c r="R40" s="18"/>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>4</v>
       </c>
@@ -2653,8 +3566,11 @@
         <f>K41*L41*M41*N41</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P41" s="18"/>
+      <c r="Q41" s="18"/>
+      <c r="R41" s="18"/>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>6</v>
       </c>
@@ -2685,8 +3601,11 @@
         <f>K42*L42*M42*N42</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P42" s="18"/>
+      <c r="Q42" s="18"/>
+      <c r="R42" s="18"/>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>11</v>
       </c>
@@ -2714,8 +3633,11 @@
         <f>K43*L43*M43*N43</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P43" s="18"/>
+      <c r="Q43" s="18"/>
+      <c r="R43" s="18"/>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>14</v>
       </c>
@@ -2743,8 +3665,11 @@
         <f>K44*L44*M44*N44</f>
         <v>15</v>
       </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P44" s="18"/>
+      <c r="Q44" s="18"/>
+      <c r="R44" s="18"/>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>16</v>
       </c>
@@ -2775,8 +3700,11 @@
         <f>K45*L45*M45*N45</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P45" s="18"/>
+      <c r="Q45" s="18"/>
+      <c r="R45" s="18"/>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>17</v>
       </c>
@@ -2804,8 +3732,11 @@
         <f>K46*L46*M46*N46</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P46" s="18"/>
+      <c r="Q46" s="18"/>
+      <c r="R46" s="18"/>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>20</v>
       </c>
@@ -2833,8 +3764,11 @@
         <f>K47*L47*M47*N47</f>
         <v>80</v>
       </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P47" s="18"/>
+      <c r="Q47" s="18"/>
+      <c r="R47" s="18"/>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>21</v>
       </c>
@@ -2862,8 +3796,11 @@
         <f>K48*L48*M48*N48</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P48" s="18"/>
+      <c r="Q48" s="18"/>
+      <c r="R48" s="18"/>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>22</v>
       </c>
@@ -2891,8 +3828,11 @@
         <f>K49*L49*M49*N49</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P49" s="18"/>
+      <c r="Q49" s="18"/>
+      <c r="R49" s="18"/>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>23</v>
       </c>
@@ -2920,8 +3860,11 @@
         <f>K50*L50*M50*N50</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P50" s="18"/>
+      <c r="Q50" s="18"/>
+      <c r="R50" s="18"/>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>24</v>
       </c>
@@ -2949,8 +3892,11 @@
         <f>K51*L51*M51*N51</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P51" s="18"/>
+      <c r="Q51" s="18"/>
+      <c r="R51" s="18"/>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>26</v>
       </c>
@@ -2978,8 +3924,11 @@
         <f>K52*L52*M52*N52</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P52" s="18"/>
+      <c r="Q52" s="18"/>
+      <c r="R52" s="18"/>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>27</v>
       </c>
@@ -3007,8 +3956,11 @@
         <f>K53*L53*M53*N53</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P53" s="18"/>
+      <c r="Q53" s="18"/>
+      <c r="R53" s="18"/>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>28</v>
       </c>
@@ -3036,8 +3988,11 @@
         <f>K54*L54*M54*N54</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P54" s="18"/>
+      <c r="Q54" s="18"/>
+      <c r="R54" s="18"/>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>29</v>
       </c>
@@ -3065,8 +4020,11 @@
         <f>K55*L55*M55*N55</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P55" s="18"/>
+      <c r="Q55" s="18"/>
+      <c r="R55" s="18"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>32</v>
       </c>
@@ -3094,8 +4052,11 @@
         <f>K56*L56*M56*N56</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P56" s="18"/>
+      <c r="Q56" s="18"/>
+      <c r="R56" s="18"/>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>33</v>
       </c>
@@ -3123,8 +4084,11 @@
         <f>K57*L57*M57*N57</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P57" s="18"/>
+      <c r="Q57" s="18"/>
+      <c r="R57" s="18"/>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>34</v>
       </c>
@@ -3155,8 +4119,11 @@
         <f>K58*L58*M58*N58</f>
         <v>198</v>
       </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P58" s="18"/>
+      <c r="Q58" s="18"/>
+      <c r="R58" s="18"/>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>35</v>
       </c>
@@ -3187,8 +4154,11 @@
         <f>K59*L59*M59*N59</f>
         <v>198</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P59" s="18"/>
+      <c r="Q59" s="18"/>
+      <c r="R59" s="18"/>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>37</v>
       </c>
@@ -3216,8 +4186,11 @@
         <f>K60*L60*M60*N60</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P60" s="18"/>
+      <c r="Q60" s="18"/>
+      <c r="R60" s="18"/>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>40</v>
       </c>
@@ -3245,8 +4218,11 @@
         <f>K61*L61*M61*N61</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P61" s="18"/>
+      <c r="Q61" s="18"/>
+      <c r="R61" s="18"/>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>41</v>
       </c>
@@ -3274,8 +4250,11 @@
         <f>K62*L62*M62*N62</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P62" s="18"/>
+      <c r="Q62" s="18"/>
+      <c r="R62" s="18"/>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>42</v>
       </c>
@@ -3307,8 +4286,11 @@
         <f>K63*L63*M63*N63</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P63" s="18"/>
+      <c r="Q63" s="18"/>
+      <c r="R63" s="18"/>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>43</v>
       </c>
@@ -3336,8 +4318,11 @@
         <f>K64*L64*M64*N64</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P64" s="18"/>
+      <c r="Q64" s="18"/>
+      <c r="R64" s="18"/>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>44</v>
       </c>
@@ -3365,8 +4350,11 @@
         <f>K65*L65*M65*N65</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P65" s="18"/>
+      <c r="Q65" s="18"/>
+      <c r="R65" s="18"/>
+    </row>
+    <row r="66" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>47</v>
       </c>
@@ -3394,8 +4382,11 @@
         <f>K66*L66*M66*N66</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="67" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="P66" s="18"/>
+      <c r="Q66" s="18"/>
+      <c r="R66" s="18"/>
+    </row>
+    <row r="67" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>48</v>
       </c>
@@ -3423,8 +4414,11 @@
         <f>K67*L67*M67*N67</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P67" s="18"/>
+      <c r="Q67" s="18"/>
+      <c r="R67" s="18"/>
+    </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>49</v>
       </c>
@@ -3452,8 +4446,11 @@
         <f>K68*L68*M68*N68</f>
         <v>30</v>
       </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P68" s="18"/>
+      <c r="Q68" s="18"/>
+      <c r="R68" s="18"/>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A69" s="6">
         <v>51</v>
       </c>
@@ -3488,8 +4485,11 @@
         <f>K69*L69*M69*N69</f>
         <v>198</v>
       </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P69" s="18"/>
+      <c r="Q69" s="18"/>
+      <c r="R69" s="18"/>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>52</v>
       </c>
@@ -3517,8 +4517,11 @@
         <f>K70*L70*M70*N70</f>
         <v>15</v>
       </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P70" s="18"/>
+      <c r="Q70" s="18"/>
+      <c r="R70" s="18"/>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>55</v>
       </c>
@@ -3551,8 +4554,11 @@
         <f>K71*L71*M71*N71</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P71" s="25"/>
+      <c r="Q71" s="25"/>
+      <c r="R71" s="25"/>
+    </row>
+    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>59</v>
       </c>
@@ -3579,16 +4585,19 @@
         <f>K72*L72*M72*N72</f>
         <v>20</v>
       </c>
+      <c r="P72" s="25"/>
+      <c r="Q72" s="25"/>
+      <c r="R72" s="25"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T61" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O72">
-      <sortCondition ref="C1:C61"/>
+  <autoFilter ref="A1:U72" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U72">
+      <sortCondition ref="Q1:Q72"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="L2">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="1"/>
         <cfvo type="num" val="2"/>
@@ -3599,16 +4608,27 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S38">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>$S2="L"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$S2="H"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>$S2="-"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="H18" r:id="rId1" tooltip="otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" xr:uid="{DC8291FA-BBBC-4164-AFDF-A14D5C37779A}"/>
-    <hyperlink ref="H28" r:id="rId2" tooltip="otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" xr:uid="{DA695823-06F7-4C4D-A0BB-56A71E8AB3AA}"/>
+    <hyperlink ref="H8" r:id="rId1" tooltip="otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.001_BriefAnalysis-TapiIetfModelLinkage.pptx" xr:uid="{DC8291FA-BBBC-4164-AFDF-A14D5C37779A}"/>
+    <hyperlink ref="H13" r:id="rId2" tooltip="otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2024.ND.002_SpotlightAndSnapshotStreams.pptx" xr:uid="{DA695823-06F7-4C4D-A0BB-56A71E8AB3AA}"/>
     <hyperlink ref="H63" r:id="rId3" tooltip="otcc2023.ND.007_BasicPhysicalIntent.zip" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2023.ND.007_BasicPhysicalIntent.zip" xr:uid="{73726784-3406-4A32-9F90-250F1899557B}"/>
-    <hyperlink ref="H17" r:id="rId4" tooltip="otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" xr:uid="{B1E96811-E3AB-4B6A-9B71-389668390DD1}"/>
-    <hyperlink ref="H26" r:id="rId5" xr:uid="{39007AE4-376B-4AFF-B690-2B1FD75ED6B2}"/>
-    <hyperlink ref="H27" r:id="rId6" xr:uid="{B85E8F47-7893-459C-8DC1-8BC4AA02A23B}"/>
-    <hyperlink ref="H29" r:id="rId7" xr:uid="{E38CDBF1-9601-4855-8DFD-AE8A6A3AD6BE}"/>
-    <hyperlink ref="H34" r:id="rId8" xr:uid="{D578898C-48FA-4D82-82AF-E6661888BC34}"/>
-    <hyperlink ref="H4" r:id="rId9" xr:uid="{09D95B53-BA52-41E5-AAC0-0F3CBDC9FC82}"/>
+    <hyperlink ref="H18" r:id="rId4" tooltip="otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" display="https://github.com/Open-Network-Models-and-Interfaces-ONMI/TAPI-Activities/blob/main/ContributionsForDiscussions/otcc2020.ND.010_TAPI-ConnectivityServiceComputationService.pptx" xr:uid="{B1E96811-E3AB-4B6A-9B71-389668390DD1}"/>
+    <hyperlink ref="H12" r:id="rId5" xr:uid="{39007AE4-376B-4AFF-B690-2B1FD75ED6B2}"/>
+    <hyperlink ref="H20" r:id="rId6" xr:uid="{B85E8F47-7893-459C-8DC1-8BC4AA02A23B}"/>
+    <hyperlink ref="H21" r:id="rId7" xr:uid="{E38CDBF1-9601-4855-8DFD-AE8A6A3AD6BE}"/>
+    <hyperlink ref="H23" r:id="rId8" xr:uid="{D578898C-48FA-4D82-82AF-E6661888BC34}"/>
+    <hyperlink ref="H2" r:id="rId9" xr:uid="{09D95B53-BA52-41E5-AAC0-0F3CBDC9FC82}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
As presented at TAPI 20250617
</commit_message>
<xml_diff>
--- a/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
+++ b/ContributionsForDiscussions/FeaturesAndWorkFor2.7.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cienacorp-my.sharepoint.com/personal/ndavis_ciena_com/Documents/Documents/WorkingDocuments/BluePlanet/ApiPo/Standards/TAPI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{769F7A87-A2C2-495B-A576-ECDB50264FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4441A210-E269-46FE-83EF-6AAD39EC710C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28875" yWindow="-16380" windowWidth="29040" windowHeight="16440" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
+    <workbookView xWindow="-75" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{D3A00CA8-A9E1-4151-B235-58AE6C28BCEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$U$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$72</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="266">
   <si>
     <t>Feature</t>
   </si>
@@ -321,9 +321,6 @@
   </si>
   <si>
     <t>Work under way in IETF. May cause changes in 2.7.</t>
-  </si>
-  <si>
-    <t>Work under way in IETF. Just for info. Will be beyond 2.7. Aim is no work in TAPI.</t>
   </si>
   <si>
     <t>Work under way in IETF. Potential future change in TAPI.</t>
@@ -779,6 +776,110 @@
   </si>
   <si>
     <t>#644</t>
+  </si>
+  <si>
+    <t>Relatively simple. 
+Brian needs to scope and provide timeline.</t>
+  </si>
+  <si>
+    <t>Next steps</t>
+  </si>
+  <si>
+    <t>BJ: Scope and timelines.</t>
+  </si>
+  <si>
+    <t>Solution identified.</t>
+  </si>
+  <si>
+    <t>Nigel to proceed with work item to make corrections to the YANG.</t>
+  </si>
+  <si>
+    <t>Action is clear.</t>
+  </si>
+  <si>
+    <t>Need to clone TR-547 for 2.5 and 2.1.3 and make string adjustments as per 2.6. This will need to be an update to the whole document, not an augment as it is a error spread throughout.</t>
+  </si>
+  <si>
+    <t>AM to identify Use Case changes</t>
+  </si>
+  <si>
+    <t>ND/AM</t>
+  </si>
+  <si>
+    <t>Proposal required</t>
+  </si>
+  <si>
+    <t>DD to propose text enhancements to RIA and any changes to YANG and/or interactions necessary to support GR.</t>
+  </si>
+  <si>
+    <t>DD has presented essence of proposal</t>
+  </si>
+  <si>
+    <t>ND discussed with Italo Busi</t>
+  </si>
+  <si>
+    <t>ND to review models.</t>
+  </si>
+  <si>
+    <t>ND to prepare contribution.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rcand ND discussed. Concluded that the issues is actually with respect to the hybrid approach of Notification. </t>
+  </si>
+  <si>
+    <t>ND to present brief contribution.</t>
+  </si>
+  <si>
+    <t>Dependent upon IETF work.</t>
+  </si>
+  <si>
+    <t>Coordination</t>
+  </si>
+  <si>
+    <t>ND: Contribution required</t>
+  </si>
+  <si>
+    <t>ND/RC: Track IETF work and extract insights as the occur.</t>
+  </si>
+  <si>
+    <t>ND: Make specific proposal in YANG.
+ND: Consider proposal for IETF model augment.</t>
+  </si>
+  <si>
+    <t>JS/ND: Connect with IETF, OC and OIF CMIS</t>
+  </si>
+  <si>
+    <t>ND to propose process…. Organic as we do work on the other issues.</t>
+  </si>
+  <si>
+    <t>ND: Formal proposal required</t>
+  </si>
+  <si>
+    <t>ND: Further detail opportunities</t>
+  </si>
+  <si>
+    <t>KK to propose change</t>
+  </si>
+  <si>
+    <t>Future</t>
+  </si>
+  <si>
+    <t>ND: Track IETF work and extract insights as the occur.</t>
+  </si>
+  <si>
+    <t>ND: Add protobuf file to 2.5.x and document.</t>
+  </si>
+  <si>
+    <t>ND to adjust TR-547</t>
+  </si>
+  <si>
+    <t>Review all properties</t>
+  </si>
+  <si>
+    <t>Propsal required.</t>
+  </si>
+  <si>
+    <t>Requires more detail.</t>
   </si>
 </sst>
 </file>
@@ -865,7 +966,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -920,6 +1021,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39994506668294322"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39994506668294322"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -962,7 +1075,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1034,7 +1147,10 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1399,7 +1515,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:U72"/>
+  <dimension ref="A1:V72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -1410,22 +1526,22 @@
     <col min="6" max="6" width="9.140625" style="1"/>
     <col min="7" max="7" width="23.5703125" style="1" customWidth="1"/>
     <col min="8" max="8" width="51.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="40.85546875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" style="1" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="15.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="18" style="1" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="10.85546875" style="1" customWidth="1"/>
-    <col min="16" max="17" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="14.5703125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="31" style="1" customWidth="1"/>
-    <col min="21" max="21" width="20.140625" style="1" customWidth="1"/>
-    <col min="22" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="10" width="18.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="40.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="18" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="10.85546875" style="1" customWidth="1"/>
+    <col min="17" max="18" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.42578125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="14.5703125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="31" style="1" customWidth="1"/>
+    <col min="22" max="22" width="20.140625" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
@@ -1433,13 +1549,13 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>56</v>
@@ -1448,49 +1564,52 @@
         <v>78</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q1" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="R1" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="S1" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P1" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="Q1" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="R1" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="S1" s="1" t="s">
+      <c r="V1" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="T1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="U1" s="17" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>15</v>
       </c>
@@ -1504,7 +1623,7 @@
         <v>2.7</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>57</v>
@@ -1513,42 +1632,47 @@
         <v>79</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="I2" s="10"/>
-      <c r="J2" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K2" s="1">
-        <v>1</v>
+        <v>125</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>236</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="L2" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M2" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N2" s="1">
         <v>1</v>
       </c>
       <c r="O2" s="1">
-        <f>K2*L2*M2*N2</f>
-        <v>3</v>
-      </c>
-      <c r="P2" s="18">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="P2" s="1">
+        <f>L2*M2*N2*O2</f>
+        <v>3</v>
       </c>
       <c r="Q2" s="18">
         <v>1</v>
       </c>
-      <c r="R2" s="18"/>
-      <c r="S2" s="1" t="str">
-        <f>IF(Q2="", "?",IF(Q2="?", "?", IF(C2=Q2, "-",IF(C2&gt;Q2,"H",IF(C2&lt;Q2,"L")))))</f>
+      <c r="R2" s="18">
+        <v>1</v>
+      </c>
+      <c r="S2" s="18"/>
+      <c r="T2" s="1" t="str">
+        <f t="shared" ref="T2:T38" si="0">IF(R2="", "?",IF(R2="?", "?", IF(C2=R2, "-",IF(C2&gt;R2,"H",IF(C2&lt;R2,"L")))))</f>
         <v>-</v>
       </c>
-      <c r="T2" s="21"/>
-    </row>
-    <row r="3" spans="1:21" ht="120" x14ac:dyDescent="0.25">
+      <c r="U2" s="21"/>
+    </row>
+    <row r="3" spans="1:22" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>57</v>
       </c>
@@ -1562,123 +1686,132 @@
         <v>2.7</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1</v>
+      <c r="J3" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>232</v>
       </c>
       <c r="L3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3" s="1">
         <v>1</v>
       </c>
       <c r="O3" s="1">
-        <f>K3*L3*M3*N3</f>
-        <v>2</v>
-      </c>
-      <c r="P3" s="18">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="P3" s="1">
+        <f>L3*M3*N3*O3</f>
+        <v>2</v>
       </c>
       <c r="Q3" s="18">
         <v>1</v>
       </c>
-      <c r="R3" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="S3" s="1" t="str">
-        <f>IF(Q3="", "?",IF(Q3="?", "?", IF(C3=Q3, "-",IF(C3&gt;Q3,"H",IF(C3&lt;Q3,"L")))))</f>
+      <c r="R3" s="18">
+        <v>1</v>
+      </c>
+      <c r="S3" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="T3" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T3" s="21"/>
-    </row>
-    <row r="4" spans="1:21" ht="60" x14ac:dyDescent="0.25">
+      <c r="U3" s="21"/>
+    </row>
+    <row r="4" spans="1:22" ht="165" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>62</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C4" s="3">
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="K4" s="1">
-        <v>1</v>
+        <v>128</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="J4" s="25" t="s">
+        <v>238</v>
       </c>
       <c r="L4" s="1">
         <v>1</v>
       </c>
       <c r="M4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="1">
-        <f>K4*L4*M4*N4</f>
-        <v>2</v>
-      </c>
-      <c r="P4" s="18">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="P4" s="1">
+        <f>L4*M4*N4*O4</f>
+        <v>2</v>
       </c>
       <c r="Q4" s="18">
         <v>1</v>
       </c>
-      <c r="R4" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="S4" s="1" t="str">
-        <f>IF(Q4="", "?",IF(Q4="?", "?", IF(C4=Q4, "-",IF(C4&gt;Q4,"H",IF(C4&lt;Q4,"L")))))</f>
+      <c r="R4" s="18">
+        <v>1</v>
+      </c>
+      <c r="S4" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="T4" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T4" s="21"/>
-    </row>
-    <row r="5" spans="1:21" ht="60" x14ac:dyDescent="0.25">
+      <c r="U4" s="21"/>
+    </row>
+    <row r="5" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>63</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="3">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="K5" s="1">
-        <v>1</v>
-      </c>
       <c r="L5" s="1">
         <v>1</v>
       </c>
@@ -1689,30 +1822,33 @@
         <v>1</v>
       </c>
       <c r="O5" s="1">
-        <f>K5*L5*M5*N5</f>
-        <v>1</v>
-      </c>
-      <c r="P5" s="18">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1">
+        <f>L5*M5*N5*O5</f>
         <v>1</v>
       </c>
       <c r="Q5" s="18">
         <v>1</v>
       </c>
-      <c r="R5" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="S5" s="1" t="str">
-        <f>IF(Q5="", "?",IF(Q5="?", "?", IF(C5=Q5, "-",IF(C5&gt;Q5,"H",IF(C5&lt;Q5,"L")))))</f>
+      <c r="R5" s="18">
+        <v>1</v>
+      </c>
+      <c r="S5" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="T5" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T5" s="21"/>
-    </row>
-    <row r="6" spans="1:21" ht="105" x14ac:dyDescent="0.25">
+      <c r="U5" s="21"/>
+    </row>
+    <row r="6" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>67</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
@@ -1724,10 +1860,10 @@
         <v>53</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="K6" s="1">
-        <v>1</v>
+        <v>148</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>241</v>
       </c>
       <c r="L6" s="1">
         <v>1</v>
@@ -1739,25 +1875,28 @@
         <v>1</v>
       </c>
       <c r="O6" s="1">
-        <f>K6*L6*M6*N6</f>
-        <v>1</v>
-      </c>
-      <c r="P6" s="18">
+        <v>1</v>
+      </c>
+      <c r="P6" s="1">
+        <f>L6*M6*N6*O6</f>
         <v>1</v>
       </c>
       <c r="Q6" s="18">
         <v>1</v>
       </c>
-      <c r="R6" s="18" t="s">
-        <v>219</v>
-      </c>
-      <c r="S6" s="1" t="str">
-        <f>IF(Q6="", "?",IF(Q6="?", "?", IF(C6=Q6, "-",IF(C6&gt;Q6,"H",IF(C6&lt;Q6,"L")))))</f>
+      <c r="R6" s="18">
+        <v>1</v>
+      </c>
+      <c r="S6" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="T6" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T6" s="21"/>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="U6" s="21"/>
+    </row>
+    <row r="7" spans="1:22" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>68</v>
       </c>
@@ -1771,27 +1910,33 @@
         <v>2.7</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="P7" s="18">
-        <v>1</v>
+      <c r="I7" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>242</v>
       </c>
       <c r="Q7" s="18">
         <v>1</v>
       </c>
-      <c r="R7" s="18"/>
-      <c r="S7" s="1" t="str">
-        <f>IF(Q7="", "?",IF(Q7="?", "?", IF(C7=Q7, "-",IF(C7&gt;Q7,"H",IF(C7&lt;Q7,"L")))))</f>
+      <c r="R7" s="18">
+        <v>1</v>
+      </c>
+      <c r="S7" s="18"/>
+      <c r="T7" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="U7" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1808,21 +1953,23 @@
         <v>53</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>76</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="I8" s="10"/>
-      <c r="J8" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="K8" s="1">
-        <v>1</v>
-      </c>
       <c r="L8" s="1">
         <v>1</v>
       </c>
@@ -1833,25 +1980,28 @@
         <v>1</v>
       </c>
       <c r="O8" s="1">
-        <f>K8*L8*M8*N8</f>
-        <v>1</v>
-      </c>
-      <c r="P8" s="18">
+        <v>1</v>
+      </c>
+      <c r="P8" s="1">
+        <f t="shared" ref="P8:P13" si="1">L8*M8*N8*O8</f>
         <v>1</v>
       </c>
       <c r="Q8" s="18">
         <v>1</v>
       </c>
-      <c r="R8" s="18"/>
-      <c r="S8" s="1" t="str">
-        <f>IF(Q8="", "?",IF(Q8="?", "?", IF(C8=Q8, "-",IF(C8&gt;Q8,"H",IF(C8&lt;Q8,"L")))))</f>
+      <c r="R8" s="18">
+        <v>1</v>
+      </c>
+      <c r="S8" s="18"/>
+      <c r="T8" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>H</v>
       </c>
-      <c r="T8" s="21" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="U8" s="21" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>9</v>
       </c>
@@ -1868,46 +2018,49 @@
         <v>53</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="K9" s="1">
-        <v>1</v>
-      </c>
       <c r="L9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="1">
         <v>1</v>
       </c>
       <c r="O9" s="1">
-        <f>K9*L9*M9*N9</f>
-        <v>2</v>
-      </c>
-      <c r="P9" s="18">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="P9" s="1">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="Q9" s="18">
         <v>1</v>
       </c>
-      <c r="R9" s="18"/>
-      <c r="S9" s="1" t="str">
-        <f>IF(Q9="", "?",IF(Q9="?", "?", IF(C9=Q9, "-",IF(C9&gt;Q9,"H",IF(C9&lt;Q9,"L")))))</f>
+      <c r="R9" s="18">
+        <v>1</v>
+      </c>
+      <c r="S9" s="18"/>
+      <c r="T9" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>H</v>
       </c>
-      <c r="T9" s="21" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="U9" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>30</v>
       </c>
@@ -1924,51 +2077,54 @@
         <v>86</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K10" s="1">
-        <v>1</v>
+      <c r="J10" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="L10" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M10" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="1">
         <v>1</v>
       </c>
       <c r="O10" s="1">
-        <f>K10*L10*M10*N10</f>
-        <v>3</v>
-      </c>
-      <c r="P10" s="22">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="P10" s="1">
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="Q10" s="22">
         <v>1</v>
       </c>
-      <c r="R10" s="22" t="s">
+      <c r="R10" s="22">
+        <v>1</v>
+      </c>
+      <c r="S10" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="T10" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>H</v>
+      </c>
+      <c r="U10" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="S10" s="1" t="str">
-        <f>IF(Q10="", "?",IF(Q10="?", "?", IF(C10=Q10, "-",IF(C10&gt;Q10,"H",IF(C10&lt;Q10,"L")))))</f>
-        <v>H</v>
-      </c>
-      <c r="T10" s="2" t="s">
+      <c r="V10" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="U10" s="1" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:22" ht="105" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>31</v>
       </c>
@@ -1990,43 +2146,49 @@
       <c r="G11" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="I11" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="J11" s="25" t="s">
+        <v>248</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="K11" s="1">
-        <v>1</v>
-      </c>
       <c r="L11" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M11" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="1">
         <v>1</v>
       </c>
       <c r="O11" s="1">
-        <f>K11*L11*M11*N11</f>
-        <v>3</v>
-      </c>
-      <c r="P11" s="18">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="P11" s="1">
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="Q11" s="18">
         <v>1</v>
       </c>
-      <c r="R11" s="18" t="s">
+      <c r="R11" s="18">
+        <v>1</v>
+      </c>
+      <c r="S11" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="T11" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>H</v>
+      </c>
+      <c r="U11" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="S11" s="1" t="str">
-        <f>IF(Q11="", "?",IF(Q11="?", "?", IF(C11=Q11, "-",IF(C11&gt;Q11,"H",IF(C11&lt;Q11,"L")))))</f>
-        <v>H</v>
-      </c>
-      <c r="T11" s="21" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" ht="225" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:22" ht="225" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>5</v>
       </c>
@@ -2040,58 +2202,63 @@
         <v>2.7</v>
       </c>
       <c r="E12" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>225</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="I12" s="11"/>
-      <c r="J12" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="J12" s="25" t="s">
+        <v>252</v>
+      </c>
+      <c r="K12" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="K12" s="1">
-        <v>1</v>
-      </c>
       <c r="L12" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M12" s="1">
+        <v>2</v>
+      </c>
+      <c r="N12" s="1">
         <v>0</v>
       </c>
-      <c r="N12" s="1">
-        <v>1</v>
-      </c>
       <c r="O12" s="1">
-        <f>K12*L12*M12*N12</f>
+        <v>1</v>
+      </c>
+      <c r="P12" s="1">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P12" s="20">
-        <v>1</v>
-      </c>
       <c r="Q12" s="20">
         <v>1</v>
       </c>
-      <c r="R12" s="20" t="s">
+      <c r="R12" s="20">
+        <v>1</v>
+      </c>
+      <c r="S12" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="T12" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>H</v>
+      </c>
+      <c r="U12" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="S12" s="1" t="str">
-        <f>IF(Q12="", "?",IF(Q12="?", "?", IF(C12=Q12, "-",IF(C12&gt;Q12,"H",IF(C12&lt;Q12,"L")))))</f>
-        <v>H</v>
-      </c>
-      <c r="T12" s="21" t="s">
+      <c r="V12" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="U12" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:22" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>10</v>
       </c>
@@ -2108,58 +2275,61 @@
         <v>53</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>76</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I13" s="10"/>
-      <c r="J13" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="K13" s="1">
-        <v>1</v>
+      <c r="J13" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="L13" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M13" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="1">
         <v>1</v>
       </c>
       <c r="O13" s="1">
-        <f>K13*L13*M13*N13</f>
-        <v>3</v>
-      </c>
-      <c r="P13" s="18">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="P13" s="1">
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="Q13" s="18">
         <v>1</v>
       </c>
-      <c r="R13" s="18" t="s">
+      <c r="R13" s="18">
+        <v>1</v>
+      </c>
+      <c r="S13" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="T13" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>H</v>
+      </c>
+      <c r="U13" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="S13" s="1" t="str">
-        <f>IF(Q13="", "?",IF(Q13="?", "?", IF(C13=Q13, "-",IF(C13&gt;Q13,"H",IF(C13&lt;Q13,"L")))))</f>
-        <v>H</v>
-      </c>
-      <c r="T13" s="21" t="s">
-        <v>189</v>
-      </c>
-      <c r="U13" s="6"/>
-    </row>
-    <row r="14" spans="1:21" ht="90" x14ac:dyDescent="0.25">
+      <c r="V13" s="6"/>
+    </row>
+    <row r="14" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>69</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C14" s="3">
         <v>3</v>
@@ -2168,35 +2338,41 @@
         <v>2.7</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="P14" s="20">
-        <v>1</v>
-      </c>
       <c r="Q14" s="20">
         <v>1</v>
       </c>
-      <c r="R14" s="24" t="s">
+      <c r="R14" s="20">
+        <v>1</v>
+      </c>
+      <c r="S14" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="T14" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>H</v>
+      </c>
+      <c r="U14" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="S14" s="1" t="str">
-        <f>IF(Q14="", "?",IF(Q14="?", "?", IF(C14=Q14, "-",IF(C14&gt;Q14,"H",IF(C14&lt;Q14,"L")))))</f>
-        <v>H</v>
-      </c>
-      <c r="T14" s="21" t="s">
+      <c r="V14" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="U14" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" ht="150" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:22" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>58</v>
       </c>
@@ -2210,105 +2386,111 @@
         <v>2.7</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="K15" s="1">
-        <v>1</v>
+      <c r="J15" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="L15" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M15" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N15" s="1">
         <v>1</v>
       </c>
       <c r="O15" s="1">
-        <f>K15*L15*M15*N15</f>
-        <v>2</v>
-      </c>
-      <c r="P15" s="18">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="P15" s="1">
+        <f t="shared" ref="P15:P34" si="2">L15*M15*N15*O15</f>
+        <v>2</v>
       </c>
       <c r="Q15" s="18">
-        <v>2</v>
-      </c>
-      <c r="R15" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="S15" s="1" t="str">
-        <f>IF(Q15="", "?",IF(Q15="?", "?", IF(C15=Q15, "-",IF(C15&gt;Q15,"H",IF(C15&lt;Q15,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R15" s="18">
+        <v>2</v>
+      </c>
+      <c r="S15" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="T15" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>L</v>
       </c>
-      <c r="T15" s="21" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" ht="60" x14ac:dyDescent="0.25">
+      <c r="U15" s="21" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>64</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C16" s="3">
         <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K16" s="1">
-        <v>1</v>
+        <v>137</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>255</v>
       </c>
       <c r="L16" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M16" s="1">
         <v>2</v>
       </c>
       <c r="N16" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16" s="1">
-        <f>K16*L16*M16*N16</f>
+        <v>1</v>
+      </c>
+      <c r="P16" s="1">
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="P16" s="18">
-        <v>3</v>
-      </c>
       <c r="Q16" s="18">
-        <v>2</v>
-      </c>
-      <c r="R16" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="R16" s="18">
+        <v>2</v>
+      </c>
+      <c r="S16" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="T16" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>L</v>
+      </c>
+      <c r="U16" s="23" t="s">
         <v>214</v>
       </c>
-      <c r="S16" s="1" t="str">
-        <f>IF(Q16="", "?",IF(Q16="?", "?", IF(C16=Q16, "-",IF(C16&gt;Q16,"H",IF(C16&lt;Q16,"L")))))</f>
-        <v>L</v>
-      </c>
-      <c r="T16" s="23" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>66</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C17" s="3">
         <v>1</v>
@@ -2320,13 +2502,13 @@
         <v>53</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="K17" s="1">
-        <v>1</v>
+        <v>145</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>256</v>
       </c>
       <c r="L17" s="1">
         <v>1</v>
@@ -2338,27 +2520,30 @@
         <v>1</v>
       </c>
       <c r="O17" s="1">
-        <f>K17*L17*M17*N17</f>
-        <v>1</v>
-      </c>
-      <c r="P17" s="18">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="P17" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
       </c>
       <c r="Q17" s="18">
-        <v>2</v>
-      </c>
-      <c r="R17" s="18" t="s">
-        <v>218</v>
-      </c>
-      <c r="S17" s="1" t="str">
-        <f>IF(Q17="", "?",IF(Q17="?", "?", IF(C17=Q17, "-",IF(C17&gt;Q17,"H",IF(C17&lt;Q17,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R17" s="18">
+        <v>2</v>
+      </c>
+      <c r="S17" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="T17" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>L</v>
       </c>
-      <c r="T17" s="23" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" ht="75" x14ac:dyDescent="0.25">
+      <c r="U17" s="23" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>2</v>
       </c>
@@ -2375,55 +2560,58 @@
         <v>53</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>81</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I18" s="10"/>
-      <c r="J18" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K18" s="1">
-        <v>1</v>
+      <c r="J18" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>159</v>
       </c>
       <c r="L18" s="1">
+        <v>1</v>
+      </c>
+      <c r="M18" s="1">
         <v>4</v>
       </c>
-      <c r="M18" s="1">
-        <v>1</v>
-      </c>
       <c r="N18" s="1">
         <v>1</v>
       </c>
       <c r="O18" s="1">
-        <f>K18*L18*M18*N18</f>
+        <v>1</v>
+      </c>
+      <c r="P18" s="1">
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="P18" s="18">
-        <v>3</v>
-      </c>
       <c r="Q18" s="18">
-        <v>2</v>
-      </c>
-      <c r="R18" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="R18" s="18">
+        <v>2</v>
+      </c>
+      <c r="S18" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="T18" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="U18" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="S18" s="1" t="str">
-        <f>IF(Q18="", "?",IF(Q18="?", "?", IF(C18=Q18, "-",IF(C18&gt;Q18,"H",IF(C18&lt;Q18,"L")))))</f>
-        <v>-</v>
-      </c>
-      <c r="T18" s="19" t="s">
+      <c r="V18" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="U18" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>53</v>
       </c>
@@ -2437,48 +2625,51 @@
         <v>2.7</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K19" s="1">
-        <v>1</v>
+      <c r="J19" s="2" t="s">
+        <v>258</v>
       </c>
       <c r="L19" s="1">
         <v>1</v>
       </c>
       <c r="M19" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N19" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" s="1">
-        <f>K19*L19*M19*N19</f>
-        <v>2</v>
-      </c>
-      <c r="P19" s="18">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="P19" s="1">
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
       <c r="Q19" s="18">
-        <v>2</v>
-      </c>
-      <c r="R19" s="18"/>
-      <c r="S19" s="1" t="str">
-        <f>IF(Q19="", "?",IF(Q19="?", "?", IF(C19=Q19, "-",IF(C19&gt;Q19,"H",IF(C19&lt;Q19,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R19" s="18">
+        <v>2</v>
+      </c>
+      <c r="S19" s="18"/>
+      <c r="T19" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T19" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="U19" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>8</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C20" s="3">
         <v>3</v>
@@ -2490,50 +2681,52 @@
         <v>53</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="I20" s="11"/>
-      <c r="J20" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="K20" s="1">
-        <v>3</v>
+        <v>121</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="J20" s="25" t="s">
+        <v>260</v>
       </c>
       <c r="L20" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M20" s="1">
+        <v>2</v>
+      </c>
+      <c r="N20" s="1">
         <v>0</v>
       </c>
-      <c r="N20" s="1">
-        <v>1</v>
-      </c>
       <c r="O20" s="1">
-        <f>K20*L20*M20*N20</f>
+        <v>1</v>
+      </c>
+      <c r="P20" s="1">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P20" s="18">
-        <v>3</v>
-      </c>
       <c r="Q20" s="18">
-        <v>2</v>
-      </c>
-      <c r="R20" s="18"/>
-      <c r="S20" s="1" t="str">
-        <f>IF(Q20="", "?",IF(Q20="?", "?", IF(C20=Q20, "-",IF(C20&gt;Q20,"H",IF(C20&lt;Q20,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R20" s="18">
+        <v>2</v>
+      </c>
+      <c r="S20" s="18"/>
+      <c r="T20" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>H</v>
       </c>
-      <c r="T20" s="21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="U20" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>12</v>
       </c>
@@ -2550,52 +2743,57 @@
         <v>53</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="I21" s="11"/>
-      <c r="J21" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="J21" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="K21" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="K21" s="1">
-        <v>1</v>
-      </c>
       <c r="L21" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M21" s="1">
+        <v>2</v>
+      </c>
+      <c r="N21" s="1">
         <v>0</v>
       </c>
-      <c r="N21" s="1">
-        <v>1</v>
-      </c>
       <c r="O21" s="1">
-        <f>K21*L21*M21*N21</f>
+        <v>1</v>
+      </c>
+      <c r="P21" s="1">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P21" s="18">
-        <v>3</v>
-      </c>
       <c r="Q21" s="18">
-        <v>2</v>
-      </c>
-      <c r="R21" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="R21" s="18">
+        <v>2</v>
+      </c>
+      <c r="S21" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="T21" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>H</v>
+      </c>
+      <c r="U21" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="S21" s="1" t="str">
-        <f>IF(Q21="", "?",IF(Q21="?", "?", IF(C21=Q21, "-",IF(C21&gt;Q21,"H",IF(C21&lt;Q21,"L")))))</f>
-        <v>H</v>
-      </c>
-      <c r="T21" s="21" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>13</v>
       </c>
@@ -2612,48 +2810,51 @@
         <v>53</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="K22" s="1">
-        <v>2</v>
+        <v>103</v>
+      </c>
+      <c r="J22" s="25" t="s">
+        <v>259</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="L22" s="1">
         <v>2</v>
       </c>
       <c r="M22" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N22" s="1">
         <v>1</v>
       </c>
       <c r="O22" s="1">
-        <f>K22*L22*M22*N22</f>
+        <v>1</v>
+      </c>
+      <c r="P22" s="1">
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="P22" s="18">
-        <v>3</v>
-      </c>
       <c r="Q22" s="18">
-        <v>2</v>
-      </c>
-      <c r="R22" s="18" t="s">
-        <v>192</v>
-      </c>
-      <c r="S22" s="1" t="str">
-        <f>IF(Q22="", "?",IF(Q22="?", "?", IF(C22=Q22, "-",IF(C22&gt;Q22,"H",IF(C22&lt;Q22,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R22" s="18">
+        <v>2</v>
+      </c>
+      <c r="S22" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="T22" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>H</v>
       </c>
-      <c r="T22" s="21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" ht="75" x14ac:dyDescent="0.25">
+      <c r="U22" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>38</v>
       </c>
@@ -2670,52 +2871,57 @@
         <v>53</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="I23" s="11"/>
-      <c r="J23" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="K23" s="1">
-        <v>2</v>
+        <v>124</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="J23" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="L23" s="1">
         <v>2</v>
       </c>
       <c r="M23" s="1">
+        <v>2</v>
+      </c>
+      <c r="N23" s="1">
         <v>0</v>
       </c>
-      <c r="N23" s="1">
-        <v>1</v>
-      </c>
       <c r="O23" s="1">
-        <f>K23*L23*M23*N23</f>
+        <v>1</v>
+      </c>
+      <c r="P23" s="1">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P23" s="18">
-        <v>3</v>
-      </c>
       <c r="Q23" s="18">
-        <v>2</v>
-      </c>
-      <c r="R23" s="18" t="s">
-        <v>202</v>
-      </c>
-      <c r="S23" s="1" t="str">
-        <f>IF(Q23="", "?",IF(Q23="?", "?", IF(C23=Q23, "-",IF(C23&gt;Q23,"H",IF(C23&lt;Q23,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R23" s="18">
+        <v>2</v>
+      </c>
+      <c r="S23" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="T23" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>H</v>
       </c>
-      <c r="T23" s="21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="U23" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>39</v>
       </c>
@@ -2732,51 +2938,56 @@
         <v>53</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K24" s="1">
-        <v>2</v>
+      <c r="I24" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="J24" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="L24" s="1">
         <v>2</v>
       </c>
       <c r="M24" s="1">
+        <v>2</v>
+      </c>
+      <c r="N24" s="1">
         <v>0</v>
       </c>
-      <c r="N24" s="1">
-        <v>1</v>
-      </c>
       <c r="O24" s="1">
-        <f>K24*L24*M24*N24</f>
+        <v>1</v>
+      </c>
+      <c r="P24" s="1">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P24" s="18">
-        <v>3</v>
-      </c>
       <c r="Q24" s="18">
-        <v>2</v>
-      </c>
-      <c r="R24" s="18" t="s">
-        <v>202</v>
-      </c>
-      <c r="S24" s="1" t="str">
-        <f>IF(Q24="", "?",IF(Q24="?", "?", IF(C24=Q24, "-",IF(C24&gt;Q24,"H",IF(C24&lt;Q24,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R24" s="18">
+        <v>2</v>
+      </c>
+      <c r="S24" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="T24" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>H</v>
       </c>
-      <c r="T24" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="U24" s="1"/>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="U24" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="V24" s="1"/>
+    </row>
+    <row r="25" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>56</v>
       </c>
@@ -2790,46 +3001,52 @@
         <v>2.7</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="K25" s="1">
-        <v>1</v>
+      <c r="I25" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="J25" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="L25" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M25" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N25" s="1">
         <v>1</v>
       </c>
       <c r="O25" s="1">
-        <f>K25*L25*M25*N25</f>
-        <v>2</v>
-      </c>
-      <c r="P25" s="18">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="P25" s="1">
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
       <c r="Q25" s="18">
-        <v>2</v>
-      </c>
-      <c r="R25" s="18"/>
-      <c r="S25" s="1" t="str">
-        <f>IF(Q25="", "?",IF(Q25="?", "?", IF(C25=Q25, "-",IF(C25&gt;Q25,"H",IF(C25&lt;Q25,"L")))))</f>
+        <v>3</v>
+      </c>
+      <c r="R25" s="18">
+        <v>2</v>
+      </c>
+      <c r="S25" s="18"/>
+      <c r="T25" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>H</v>
       </c>
-      <c r="T25" s="21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" ht="60" x14ac:dyDescent="0.25">
+      <c r="U25" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>18</v>
       </c>
@@ -2846,48 +3063,51 @@
         <v>53</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J26" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="J26" s="26" t="s">
+        <v>263</v>
+      </c>
+      <c r="K26" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="K26" s="1">
-        <v>1</v>
-      </c>
       <c r="L26" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M26" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N26" s="1">
         <v>1</v>
       </c>
       <c r="O26" s="1">
-        <f>K26*L26*M26*N26</f>
-        <v>2</v>
-      </c>
-      <c r="P26" s="18">
+        <v>1</v>
+      </c>
+      <c r="P26" s="1">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="Q26" s="18">
         <v>5</v>
       </c>
-      <c r="Q26" s="18">
-        <v>3</v>
-      </c>
-      <c r="R26" s="18" t="s">
+      <c r="R26" s="18">
+        <v>3</v>
+      </c>
+      <c r="S26" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="T26" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>L</v>
+      </c>
+      <c r="U26" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="S26" s="1" t="str">
-        <f>IF(Q26="", "?",IF(Q26="?", "?", IF(C26=Q26, "-",IF(C26&gt;Q26,"H",IF(C26&lt;Q26,"L")))))</f>
-        <v>L</v>
-      </c>
-      <c r="T26" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:22" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>54</v>
       </c>
@@ -2898,7 +3118,7 @@
         <v>1</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>53</v>
@@ -2906,100 +3126,106 @@
       <c r="F27" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="J27" s="1" t="s">
+      <c r="J27" s="26" t="s">
+        <v>263</v>
+      </c>
+      <c r="K27" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="K27" s="1">
-        <v>1</v>
-      </c>
       <c r="L27" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M27" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N27" s="1">
         <v>1</v>
       </c>
       <c r="O27" s="1">
-        <f>K27*L27*M27*N27</f>
-        <v>2</v>
-      </c>
-      <c r="P27" s="18">
+        <v>1</v>
+      </c>
+      <c r="P27" s="1">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="Q27" s="18">
         <v>5</v>
       </c>
-      <c r="Q27" s="18">
-        <v>3</v>
-      </c>
-      <c r="R27" s="18" t="s">
-        <v>193</v>
-      </c>
-      <c r="S27" s="1" t="str">
-        <f>IF(Q27="", "?",IF(Q27="?", "?", IF(C27=Q27, "-",IF(C27&gt;Q27,"H",IF(C27&lt;Q27,"L")))))</f>
+      <c r="R27" s="18">
+        <v>3</v>
+      </c>
+      <c r="S27" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="T27" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>L</v>
       </c>
-      <c r="T27" s="23" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="U27" s="23" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>61</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C28" s="3">
         <v>1</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>53</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="K28" s="1">
-        <v>1</v>
+        <v>127</v>
+      </c>
+      <c r="J28" s="25" t="s">
+        <v>262</v>
       </c>
       <c r="L28" s="1">
         <v>1</v>
       </c>
       <c r="M28" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N28" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O28" s="1">
-        <f>K28*L28*M28*N28</f>
-        <v>2</v>
-      </c>
-      <c r="P28" s="18">
+        <v>1</v>
+      </c>
+      <c r="P28" s="1">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="Q28" s="18">
         <v>5</v>
       </c>
-      <c r="Q28" s="18">
-        <v>3</v>
-      </c>
-      <c r="R28" s="18" t="s">
-        <v>211</v>
-      </c>
-      <c r="S28" s="1" t="str">
-        <f>IF(Q28="", "?",IF(Q28="?", "?", IF(C28=Q28, "-",IF(C28&gt;Q28,"H",IF(C28&lt;Q28,"L")))))</f>
+      <c r="R28" s="18">
+        <v>3</v>
+      </c>
+      <c r="S28" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="T28" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>L</v>
       </c>
-      <c r="T28" s="23" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="U28" s="23" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>65</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C29" s="3">
         <v>1</v>
@@ -3011,10 +3237,13 @@
         <v>53</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="K29" s="1">
-        <v>1</v>
+        <v>140</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>261</v>
       </c>
       <c r="L29" s="1">
         <v>1</v>
@@ -3026,27 +3255,30 @@
         <v>1</v>
       </c>
       <c r="O29" s="1">
-        <f>K29*L29*M29*N29</f>
-        <v>1</v>
-      </c>
-      <c r="P29" s="18">
+        <v>1</v>
+      </c>
+      <c r="P29" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="Q29" s="18">
         <v>5</v>
       </c>
-      <c r="Q29" s="18">
-        <v>3</v>
-      </c>
-      <c r="R29" s="18" t="s">
+      <c r="R29" s="18">
+        <v>3</v>
+      </c>
+      <c r="S29" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="T29" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>L</v>
+      </c>
+      <c r="U29" s="23" t="s">
         <v>216</v>
       </c>
-      <c r="S29" s="1" t="str">
-        <f>IF(Q29="", "?",IF(Q29="?", "?", IF(C29=Q29, "-",IF(C29&gt;Q29,"H",IF(C29&lt;Q29,"L")))))</f>
-        <v>L</v>
-      </c>
-      <c r="T29" s="23" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>25</v>
       </c>
@@ -3065,41 +3297,41 @@
       <c r="G30" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K30" s="1">
-        <v>3</v>
+      <c r="K30" s="1" t="s">
+        <v>109</v>
       </c>
       <c r="L30" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M30" s="1">
+        <v>2</v>
+      </c>
+      <c r="N30" s="1">
         <v>0</v>
       </c>
-      <c r="N30" s="1">
-        <v>1</v>
-      </c>
       <c r="O30" s="1">
-        <f>K30*L30*M30*N30</f>
+        <v>1</v>
+      </c>
+      <c r="P30" s="1">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P30" s="18">
+      <c r="Q30" s="18">
         <v>5</v>
       </c>
-      <c r="Q30" s="18">
-        <v>3</v>
-      </c>
-      <c r="R30" s="18"/>
-      <c r="S30" s="1" t="str">
-        <f>IF(Q30="", "?",IF(Q30="?", "?", IF(C30=Q30, "-",IF(C30&gt;Q30,"H",IF(C30&lt;Q30,"L")))))</f>
+      <c r="R30" s="18">
+        <v>3</v>
+      </c>
+      <c r="S30" s="18"/>
+      <c r="T30" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T30" s="21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="U30" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>36</v>
       </c>
@@ -3118,41 +3350,41 @@
       <c r="G31" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="K31" s="1">
-        <v>2</v>
+      <c r="K31" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="L31" s="1">
+        <v>2</v>
+      </c>
+      <c r="M31" s="1">
         <v>5</v>
       </c>
-      <c r="M31" s="1">
+      <c r="N31" s="1">
         <v>0</v>
       </c>
-      <c r="N31" s="1">
-        <v>1</v>
-      </c>
       <c r="O31" s="1">
-        <f>K31*L31*M31*N31</f>
+        <v>1</v>
+      </c>
+      <c r="P31" s="1">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P31" s="18">
+      <c r="Q31" s="18">
         <v>5</v>
       </c>
-      <c r="Q31" s="18">
-        <v>3</v>
-      </c>
-      <c r="R31" s="18"/>
-      <c r="S31" s="1" t="str">
-        <f>IF(Q31="", "?",IF(Q31="?", "?", IF(C31=Q31, "-",IF(C31&gt;Q31,"H",IF(C31&lt;Q31,"L")))))</f>
+      <c r="R31" s="18">
+        <v>3</v>
+      </c>
+      <c r="S31" s="18"/>
+      <c r="T31" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="T31" s="21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="U31" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>50</v>
       </c>
@@ -3171,43 +3403,43 @@
       <c r="G32" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="J32" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K32" s="1">
-        <v>1</v>
+      <c r="K32" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="L32" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M32" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N32" s="1">
         <v>1</v>
       </c>
       <c r="O32" s="1">
-        <f>K32*L32*M32*N32</f>
-        <v>3</v>
-      </c>
-      <c r="P32" s="18">
+        <v>1</v>
+      </c>
+      <c r="P32" s="1">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="Q32" s="18">
         <v>5</v>
       </c>
-      <c r="Q32" s="18">
-        <v>3</v>
-      </c>
-      <c r="R32" s="18" t="s">
+      <c r="R32" s="18">
+        <v>3</v>
+      </c>
+      <c r="S32" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="T32" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="U32" s="21" t="s">
         <v>205</v>
       </c>
-      <c r="S32" s="1" t="str">
-        <f>IF(Q32="", "?",IF(Q32="?", "?", IF(C32=Q32, "-",IF(C32&gt;Q32,"H",IF(C32&lt;Q32,"L")))))</f>
-        <v>-</v>
-      </c>
-      <c r="T32" s="21" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>46</v>
       </c>
@@ -3227,13 +3459,11 @@
         <v>77</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="J33" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="K33" s="1">
-        <v>1</v>
+      <c r="J33" s="12"/>
+      <c r="K33" s="1" t="s">
+        <v>167</v>
       </c>
       <c r="L33" s="1">
         <v>1</v>
@@ -3245,25 +3475,28 @@
         <v>1</v>
       </c>
       <c r="O33" s="1">
-        <f>K33*L33*M33*N33</f>
-        <v>1</v>
-      </c>
-      <c r="P33" s="22" t="s">
-        <v>147</v>
+        <v>1</v>
+      </c>
+      <c r="P33" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
       </c>
       <c r="Q33" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="R33" s="22"/>
-      <c r="S33" s="1" t="str">
-        <f>IF(Q33="", "?",IF(Q33="?", "?", IF(C33=Q33, "-",IF(C33&gt;Q33,"H",IF(C33&lt;Q33,"L")))))</f>
+        <v>146</v>
+      </c>
+      <c r="R33" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="S33" s="22"/>
+      <c r="T33" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>?</v>
       </c>
-      <c r="T33" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="U33" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>19</v>
       </c>
@@ -3279,75 +3512,76 @@
       <c r="E34" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="K34" s="1">
-        <v>1</v>
-      </c>
       <c r="L34" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M34" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N34" s="1">
         <v>1</v>
       </c>
       <c r="O34" s="1">
-        <f>K34*L34*M34*N34</f>
-        <v>3</v>
-      </c>
-      <c r="P34" s="22" t="s">
-        <v>147</v>
+        <v>1</v>
+      </c>
+      <c r="P34" s="1">
+        <f t="shared" si="2"/>
+        <v>3</v>
       </c>
       <c r="Q34" s="22" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="R34" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="S34" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="T34" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>?</v>
+      </c>
+      <c r="U34" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="S34" s="1" t="str">
-        <f>IF(Q34="", "?",IF(Q34="?", "?", IF(C34=Q34, "-",IF(C34&gt;Q34,"H",IF(C34&lt;Q34,"L")))))</f>
-        <v>?</v>
-      </c>
-      <c r="T34" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>70</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C35" s="15">
         <v>0</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F35" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I35" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="I35" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="P35" s="18"/>
+      <c r="J35" s="14"/>
       <c r="Q35" s="18"/>
       <c r="R35" s="18"/>
-      <c r="S35" s="1" t="str">
-        <f>IF(Q35="", "?",IF(Q35="?", "?", IF(C35=Q35, "-",IF(C35&gt;Q35,"H",IF(C35&lt;Q35,"L")))))</f>
+      <c r="S35" s="18"/>
+      <c r="T35" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>?</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>71</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C36" s="15">
         <v>0</v>
@@ -3356,23 +3590,24 @@
         <v>2.5</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I36" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="P36" s="18"/>
+        <v>163</v>
+      </c>
+      <c r="J36" s="14"/>
       <c r="Q36" s="18"/>
       <c r="R36" s="18"/>
-      <c r="S36" s="1" t="str">
-        <f>IF(Q36="", "?",IF(Q36="?", "?", IF(C36=Q36, "-",IF(C36&gt;Q36,"H",IF(C36&lt;Q36,"L")))))</f>
+      <c r="S36" s="18"/>
+      <c r="T36" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>?</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>45</v>
       </c>
@@ -3389,49 +3624,49 @@
         <v>86</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="J37" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="K37" s="1">
-        <v>1</v>
+      <c r="K37" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="L37" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M37" s="1">
         <v>2</v>
       </c>
       <c r="N37" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O37" s="1">
-        <f>K37*L37*M37*N37</f>
+        <v>1</v>
+      </c>
+      <c r="P37" s="1">
+        <f t="shared" ref="P37:P72" si="3">L37*M37*N37*O37</f>
         <v>4</v>
       </c>
-      <c r="P37" s="22"/>
       <c r="Q37" s="22"/>
-      <c r="R37" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="S37" s="1" t="str">
-        <f>IF(Q37="", "?",IF(Q37="?", "?", IF(C37=Q37, "-",IF(C37&gt;Q37,"H",IF(C37&lt;Q37,"L")))))</f>
+      <c r="R37" s="22"/>
+      <c r="S37" s="22" t="s">
+        <v>202</v>
+      </c>
+      <c r="T37" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>?</v>
       </c>
-      <c r="T37" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="U37" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>60</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C38" s="3">
         <v>2</v>
@@ -3442,39 +3677,39 @@
       <c r="E38" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="J38" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="K38" s="1">
-        <v>1</v>
+      <c r="K38" s="1" t="s">
+        <v>111</v>
       </c>
       <c r="L38" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M38" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N38" s="1">
         <v>1</v>
       </c>
       <c r="O38" s="1">
-        <f>K38*L38*M38*N38</f>
-        <v>3</v>
-      </c>
-      <c r="P38" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="P38" s="1">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
       <c r="Q38" s="22"/>
-      <c r="R38" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="S38" s="1" t="str">
-        <f>IF(Q38="", "?",IF(Q38="?", "?", IF(C38=Q38, "-",IF(C38&gt;Q38,"H",IF(C38&lt;Q38,"L")))))</f>
+      <c r="R38" s="22"/>
+      <c r="S38" s="22" t="s">
+        <v>202</v>
+      </c>
+      <c r="T38" s="1" t="str">
+        <f t="shared" si="0"/>
         <v>?</v>
       </c>
-      <c r="T38" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U38" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>1</v>
       </c>
@@ -3483,30 +3718,30 @@
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E39" s="5"/>
-      <c r="K39" s="1">
-        <v>2</v>
-      </c>
       <c r="L39" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M39" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N39" s="1">
+        <v>1</v>
+      </c>
+      <c r="O39" s="1">
         <v>5</v>
       </c>
-      <c r="O39" s="1">
-        <f>K39*L39*M39*N39</f>
+      <c r="P39" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P39" s="18"/>
       <c r="Q39" s="18"/>
       <c r="R39" s="18"/>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S39" s="18"/>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>3</v>
       </c>
@@ -3515,30 +3750,30 @@
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E40" s="5"/>
-      <c r="K40" s="1">
-        <v>1</v>
-      </c>
       <c r="L40" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M40" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N40" s="1">
+        <v>1</v>
+      </c>
+      <c r="O40" s="1">
         <v>5</v>
       </c>
-      <c r="O40" s="1">
-        <f>K40*L40*M40*N40</f>
+      <c r="P40" s="1">
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="P40" s="18"/>
       <c r="Q40" s="18"/>
       <c r="R40" s="18"/>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S40" s="18"/>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>4</v>
       </c>
@@ -3547,12 +3782,9 @@
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E41" s="2"/>
-      <c r="K41" s="1">
-        <v>2</v>
-      </c>
       <c r="L41" s="1">
         <v>2</v>
       </c>
@@ -3560,17 +3792,20 @@
         <v>2</v>
       </c>
       <c r="N41" s="1">
+        <v>2</v>
+      </c>
+      <c r="O41" s="1">
         <v>5</v>
       </c>
-      <c r="O41" s="1">
-        <f>K41*L41*M41*N41</f>
+      <c r="P41" s="1">
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="P41" s="18"/>
       <c r="Q41" s="18"/>
       <c r="R41" s="18"/>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S41" s="18"/>
+    </row>
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>6</v>
       </c>
@@ -3579,33 +3814,33 @@
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E42" s="5"/>
       <c r="F42" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="K42" s="1">
-        <v>2</v>
-      </c>
       <c r="L42" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M42" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N42" s="1">
+        <v>2</v>
+      </c>
+      <c r="O42" s="1">
         <v>5</v>
       </c>
-      <c r="O42" s="1">
-        <f>K42*L42*M42*N42</f>
+      <c r="P42" s="1">
+        <f t="shared" si="3"/>
         <v>60</v>
       </c>
-      <c r="P42" s="18"/>
       <c r="Q42" s="18"/>
       <c r="R42" s="18"/>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S42" s="18"/>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>11</v>
       </c>
@@ -3614,30 +3849,30 @@
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E43" s="2"/>
-      <c r="K43" s="1">
-        <v>2</v>
-      </c>
       <c r="L43" s="1">
         <v>2</v>
       </c>
       <c r="M43" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N43" s="1">
+        <v>1</v>
+      </c>
+      <c r="O43" s="1">
         <v>5</v>
       </c>
-      <c r="O43" s="1">
-        <f>K43*L43*M43*N43</f>
+      <c r="P43" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P43" s="18"/>
       <c r="Q43" s="18"/>
       <c r="R43" s="18"/>
-    </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S43" s="18"/>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>14</v>
       </c>
@@ -3646,30 +3881,30 @@
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E44" s="5"/>
-      <c r="K44" s="1">
-        <v>1</v>
-      </c>
       <c r="L44" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M44" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N44" s="1">
+        <v>1</v>
+      </c>
+      <c r="O44" s="1">
         <v>5</v>
       </c>
-      <c r="O44" s="1">
-        <f>K44*L44*M44*N44</f>
+      <c r="P44" s="1">
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="P44" s="18"/>
       <c r="Q44" s="18"/>
       <c r="R44" s="18"/>
-    </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S44" s="18"/>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>16</v>
       </c>
@@ -3678,33 +3913,33 @@
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E45" s="2"/>
-      <c r="J45" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="K45" s="1">
-        <v>2</v>
+      <c r="K45" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="L45" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M45" s="1">
         <v>1</v>
       </c>
       <c r="N45" s="1">
+        <v>1</v>
+      </c>
+      <c r="O45" s="1">
         <v>5</v>
       </c>
-      <c r="O45" s="1">
-        <f>K45*L45*M45*N45</f>
+      <c r="P45" s="1">
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="P45" s="18"/>
       <c r="Q45" s="18"/>
       <c r="R45" s="18"/>
-    </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S45" s="18"/>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>17</v>
       </c>
@@ -3713,12 +3948,9 @@
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E46" s="2"/>
-      <c r="K46" s="1">
-        <v>2</v>
-      </c>
       <c r="L46" s="1">
         <v>2</v>
       </c>
@@ -3726,17 +3958,20 @@
         <v>2</v>
       </c>
       <c r="N46" s="1">
+        <v>2</v>
+      </c>
+      <c r="O46" s="1">
         <v>5</v>
       </c>
-      <c r="O46" s="1">
-        <f>K46*L46*M46*N46</f>
+      <c r="P46" s="1">
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="P46" s="18"/>
       <c r="Q46" s="18"/>
       <c r="R46" s="18"/>
-    </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S46" s="18"/>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>20</v>
       </c>
@@ -3745,30 +3980,30 @@
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E47" s="5"/>
-      <c r="K47" s="1">
-        <v>2</v>
-      </c>
       <c r="L47" s="1">
+        <v>2</v>
+      </c>
+      <c r="M47" s="1">
         <v>4</v>
       </c>
-      <c r="M47" s="1">
-        <v>2</v>
-      </c>
       <c r="N47" s="1">
+        <v>2</v>
+      </c>
+      <c r="O47" s="1">
         <v>5</v>
       </c>
-      <c r="O47" s="1">
-        <f>K47*L47*M47*N47</f>
+      <c r="P47" s="1">
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
-      <c r="P47" s="18"/>
       <c r="Q47" s="18"/>
       <c r="R47" s="18"/>
-    </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="S47" s="18"/>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>21</v>
       </c>
@@ -3777,30 +4012,30 @@
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E48" s="2"/>
-      <c r="K48" s="1">
-        <v>2</v>
-      </c>
       <c r="L48" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M48" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N48" s="1">
+        <v>2</v>
+      </c>
+      <c r="O48" s="1">
         <v>5</v>
       </c>
-      <c r="O48" s="1">
-        <f>K48*L48*M48*N48</f>
+      <c r="P48" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P48" s="18"/>
       <c r="Q48" s="18"/>
       <c r="R48" s="18"/>
-    </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S48" s="18"/>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>22</v>
       </c>
@@ -3809,30 +4044,30 @@
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E49" s="2"/>
-      <c r="K49" s="1">
-        <v>2</v>
-      </c>
       <c r="L49" s="1">
         <v>2</v>
       </c>
       <c r="M49" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N49" s="1">
+        <v>1</v>
+      </c>
+      <c r="O49" s="1">
         <v>5</v>
       </c>
-      <c r="O49" s="1">
-        <f>K49*L49*M49*N49</f>
+      <c r="P49" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P49" s="18"/>
       <c r="Q49" s="18"/>
       <c r="R49" s="18"/>
-    </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S49" s="18"/>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>23</v>
       </c>
@@ -3841,30 +4076,30 @@
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E50" s="2"/>
-      <c r="K50" s="1">
-        <v>2</v>
-      </c>
       <c r="L50" s="1">
         <v>2</v>
       </c>
       <c r="M50" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N50" s="1">
+        <v>1</v>
+      </c>
+      <c r="O50" s="1">
         <v>5</v>
       </c>
-      <c r="O50" s="1">
-        <f>K50*L50*M50*N50</f>
+      <c r="P50" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P50" s="18"/>
       <c r="Q50" s="18"/>
       <c r="R50" s="18"/>
-    </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S50" s="18"/>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>24</v>
       </c>
@@ -3873,30 +4108,30 @@
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E51" s="5"/>
-      <c r="K51" s="1">
-        <v>2</v>
-      </c>
       <c r="L51" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M51" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N51" s="1">
+        <v>1</v>
+      </c>
+      <c r="O51" s="1">
         <v>5</v>
       </c>
-      <c r="O51" s="1">
-        <f>K51*L51*M51*N51</f>
+      <c r="P51" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P51" s="18"/>
       <c r="Q51" s="18"/>
       <c r="R51" s="18"/>
-    </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S51" s="18"/>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>26</v>
       </c>
@@ -3905,12 +4140,9 @@
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E52" s="2"/>
-      <c r="K52" s="1">
-        <v>2</v>
-      </c>
       <c r="L52" s="1">
         <v>2</v>
       </c>
@@ -3918,17 +4150,20 @@
         <v>2</v>
       </c>
       <c r="N52" s="1">
+        <v>2</v>
+      </c>
+      <c r="O52" s="1">
         <v>5</v>
       </c>
-      <c r="O52" s="1">
-        <f>K52*L52*M52*N52</f>
+      <c r="P52" s="1">
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="P52" s="18"/>
       <c r="Q52" s="18"/>
       <c r="R52" s="18"/>
-    </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S52" s="18"/>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>27</v>
       </c>
@@ -3937,30 +4172,30 @@
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E53" s="2"/>
-      <c r="K53" s="1">
-        <v>2</v>
-      </c>
       <c r="L53" s="1">
         <v>2</v>
       </c>
       <c r="M53" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N53" s="1">
+        <v>1</v>
+      </c>
+      <c r="O53" s="1">
         <v>5</v>
       </c>
-      <c r="O53" s="1">
-        <f>K53*L53*M53*N53</f>
+      <c r="P53" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P53" s="18"/>
       <c r="Q53" s="18"/>
       <c r="R53" s="18"/>
-    </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S53" s="18"/>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>28</v>
       </c>
@@ -3969,30 +4204,30 @@
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E54" s="2"/>
-      <c r="K54" s="1">
-        <v>2</v>
-      </c>
       <c r="L54" s="1">
         <v>2</v>
       </c>
       <c r="M54" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N54" s="1">
+        <v>1</v>
+      </c>
+      <c r="O54" s="1">
         <v>5</v>
       </c>
-      <c r="O54" s="1">
-        <f>K54*L54*M54*N54</f>
+      <c r="P54" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P54" s="18"/>
       <c r="Q54" s="18"/>
       <c r="R54" s="18"/>
-    </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S54" s="18"/>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>29</v>
       </c>
@@ -4001,30 +4236,30 @@
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E55" s="5"/>
-      <c r="K55" s="1">
-        <v>2</v>
-      </c>
       <c r="L55" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M55" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N55" s="1">
+        <v>1</v>
+      </c>
+      <c r="O55" s="1">
         <v>5</v>
       </c>
-      <c r="O55" s="1">
-        <f>K55*L55*M55*N55</f>
+      <c r="P55" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P55" s="18"/>
       <c r="Q55" s="18"/>
       <c r="R55" s="18"/>
-    </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S55" s="18"/>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>32</v>
       </c>
@@ -4033,30 +4268,30 @@
       </c>
       <c r="C56" s="3"/>
       <c r="D56" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E56" s="2"/>
-      <c r="K56" s="1">
-        <v>2</v>
-      </c>
       <c r="L56" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M56" s="1">
         <v>1</v>
       </c>
       <c r="N56" s="1">
+        <v>1</v>
+      </c>
+      <c r="O56" s="1">
         <v>5</v>
       </c>
-      <c r="O56" s="1">
-        <f>K56*L56*M56*N56</f>
+      <c r="P56" s="1">
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="P56" s="18"/>
       <c r="Q56" s="18"/>
       <c r="R56" s="18"/>
-    </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S56" s="18"/>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>33</v>
       </c>
@@ -4065,30 +4300,30 @@
       </c>
       <c r="C57" s="3"/>
       <c r="D57" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E57" s="5"/>
-      <c r="K57" s="1">
-        <v>2</v>
-      </c>
       <c r="L57" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M57" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N57" s="1">
+        <v>1</v>
+      </c>
+      <c r="O57" s="1">
         <v>5</v>
       </c>
-      <c r="O57" s="1">
-        <f>K57*L57*M57*N57</f>
+      <c r="P57" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P57" s="18"/>
       <c r="Q57" s="18"/>
       <c r="R57" s="18"/>
-    </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S57" s="18"/>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>34</v>
       </c>
@@ -4097,33 +4332,33 @@
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E58" s="2"/>
-      <c r="J58" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="K58" s="1">
-        <v>2</v>
+      <c r="K58" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="L58" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M58" s="1">
         <v>1</v>
       </c>
       <c r="N58" s="1">
+        <v>1</v>
+      </c>
+      <c r="O58" s="1">
         <v>99</v>
       </c>
-      <c r="O58" s="1">
-        <f>K58*L58*M58*N58</f>
+      <c r="P58" s="1">
+        <f t="shared" si="3"/>
         <v>198</v>
       </c>
-      <c r="P58" s="18"/>
       <c r="Q58" s="18"/>
       <c r="R58" s="18"/>
-    </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S58" s="18"/>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>35</v>
       </c>
@@ -4132,33 +4367,33 @@
       </c>
       <c r="C59" s="4"/>
       <c r="D59" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E59" s="2"/>
-      <c r="J59" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="K59" s="1">
-        <v>2</v>
+      <c r="K59" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="L59" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M59" s="1">
         <v>1</v>
       </c>
       <c r="N59" s="1">
+        <v>1</v>
+      </c>
+      <c r="O59" s="1">
         <v>99</v>
       </c>
-      <c r="O59" s="1">
-        <f>K59*L59*M59*N59</f>
+      <c r="P59" s="1">
+        <f t="shared" si="3"/>
         <v>198</v>
       </c>
-      <c r="P59" s="18"/>
       <c r="Q59" s="18"/>
       <c r="R59" s="18"/>
-    </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S59" s="18"/>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>37</v>
       </c>
@@ -4167,12 +4402,9 @@
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E60" s="2"/>
-      <c r="K60" s="1">
-        <v>2</v>
-      </c>
       <c r="L60" s="1">
         <v>2</v>
       </c>
@@ -4180,17 +4412,20 @@
         <v>2</v>
       </c>
       <c r="N60" s="1">
+        <v>2</v>
+      </c>
+      <c r="O60" s="1">
         <v>5</v>
       </c>
-      <c r="O60" s="1">
-        <f>K60*L60*M60*N60</f>
+      <c r="P60" s="1">
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="P60" s="18"/>
       <c r="Q60" s="18"/>
       <c r="R60" s="18"/>
-    </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S60" s="18"/>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>40</v>
       </c>
@@ -4199,30 +4434,30 @@
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E61" s="5"/>
-      <c r="K61" s="1">
-        <v>2</v>
-      </c>
       <c r="L61" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M61" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N61" s="1">
+        <v>1</v>
+      </c>
+      <c r="O61" s="1">
         <v>5</v>
       </c>
-      <c r="O61" s="1">
-        <f>K61*L61*M61*N61</f>
+      <c r="P61" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P61" s="18"/>
       <c r="Q61" s="18"/>
       <c r="R61" s="18"/>
-    </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S61" s="18"/>
+    </row>
+    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>41</v>
       </c>
@@ -4231,30 +4466,30 @@
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E62" s="5"/>
-      <c r="K62" s="1">
-        <v>2</v>
-      </c>
       <c r="L62" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M62" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N62" s="1">
+        <v>1</v>
+      </c>
+      <c r="O62" s="1">
         <v>5</v>
       </c>
-      <c r="O62" s="1">
-        <f>K62*L62*M62*N62</f>
+      <c r="P62" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P62" s="18"/>
       <c r="Q62" s="18"/>
       <c r="R62" s="18"/>
-    </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S62" s="18"/>
+    </row>
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>42</v>
       </c>
@@ -4263,34 +4498,35 @@
       </c>
       <c r="C63" s="3"/>
       <c r="D63" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E63" s="5"/>
       <c r="H63" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I63" s="10"/>
-      <c r="K63" s="1">
-        <v>2</v>
-      </c>
+      <c r="J63" s="10"/>
       <c r="L63" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M63" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N63" s="1">
+        <v>1</v>
+      </c>
+      <c r="O63" s="1">
         <v>5</v>
       </c>
-      <c r="O63" s="1">
-        <f>K63*L63*M63*N63</f>
+      <c r="P63" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P63" s="18"/>
       <c r="Q63" s="18"/>
       <c r="R63" s="18"/>
-    </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S63" s="18"/>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>43</v>
       </c>
@@ -4299,30 +4535,30 @@
       </c>
       <c r="C64" s="3"/>
       <c r="D64" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E64" s="5"/>
-      <c r="K64" s="1">
-        <v>2</v>
-      </c>
       <c r="L64" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M64" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N64" s="1">
+        <v>1</v>
+      </c>
+      <c r="O64" s="1">
         <v>5</v>
       </c>
-      <c r="O64" s="1">
-        <f>K64*L64*M64*N64</f>
+      <c r="P64" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P64" s="18"/>
       <c r="Q64" s="18"/>
       <c r="R64" s="18"/>
-    </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S64" s="18"/>
+    </row>
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>44</v>
       </c>
@@ -4331,30 +4567,30 @@
       </c>
       <c r="C65" s="3"/>
       <c r="D65" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E65" s="5"/>
-      <c r="K65" s="1">
-        <v>2</v>
-      </c>
       <c r="L65" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M65" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N65" s="1">
+        <v>1</v>
+      </c>
+      <c r="O65" s="1">
         <v>5</v>
       </c>
-      <c r="O65" s="1">
-        <f>K65*L65*M65*N65</f>
+      <c r="P65" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P65" s="18"/>
       <c r="Q65" s="18"/>
       <c r="R65" s="18"/>
-    </row>
-    <row r="66" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="S65" s="18"/>
+    </row>
+    <row r="66" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>47</v>
       </c>
@@ -4363,30 +4599,30 @@
       </c>
       <c r="C66" s="3"/>
       <c r="D66" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E66" s="2"/>
-      <c r="K66" s="1">
-        <v>2</v>
-      </c>
       <c r="L66" s="1">
         <v>2</v>
       </c>
       <c r="M66" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N66" s="1">
+        <v>1</v>
+      </c>
+      <c r="O66" s="1">
         <v>5</v>
       </c>
-      <c r="O66" s="1">
-        <f>K66*L66*M66*N66</f>
+      <c r="P66" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P66" s="18"/>
       <c r="Q66" s="18"/>
       <c r="R66" s="18"/>
-    </row>
-    <row r="67" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="S66" s="18"/>
+    </row>
+    <row r="67" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>48</v>
       </c>
@@ -4395,30 +4631,30 @@
       </c>
       <c r="C67" s="3"/>
       <c r="D67" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E67" s="5"/>
-      <c r="K67" s="1">
-        <v>2</v>
-      </c>
       <c r="L67" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M67" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N67" s="1">
+        <v>1</v>
+      </c>
+      <c r="O67" s="1">
         <v>5</v>
       </c>
-      <c r="O67" s="1">
-        <f>K67*L67*M67*N67</f>
+      <c r="P67" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P67" s="18"/>
       <c r="Q67" s="18"/>
       <c r="R67" s="18"/>
-    </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S67" s="18"/>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>49</v>
       </c>
@@ -4427,30 +4663,30 @@
       </c>
       <c r="C68" s="3"/>
       <c r="D68" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E68" s="5"/>
-      <c r="K68" s="1">
-        <v>2</v>
-      </c>
       <c r="L68" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M68" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N68" s="1">
+        <v>1</v>
+      </c>
+      <c r="O68" s="1">
         <v>5</v>
       </c>
-      <c r="O68" s="1">
-        <f>K68*L68*M68*N68</f>
+      <c r="P68" s="1">
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="P68" s="18"/>
       <c r="Q68" s="18"/>
       <c r="R68" s="18"/>
-    </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S68" s="18"/>
+    </row>
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A69" s="6">
         <v>51</v>
       </c>
@@ -4459,37 +4695,38 @@
       </c>
       <c r="C69" s="4"/>
       <c r="D69" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E69" s="7"/>
       <c r="F69" s="6"/>
       <c r="G69" s="6"/>
       <c r="H69" s="6"/>
       <c r="I69" s="6"/>
-      <c r="J69" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="K69" s="1">
-        <v>2</v>
-      </c>
-      <c r="L69" s="6">
-        <v>1</v>
+      <c r="J69" s="6"/>
+      <c r="K69" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="L69" s="1">
+        <v>2</v>
       </c>
       <c r="M69" s="6">
         <v>1</v>
       </c>
       <c r="N69" s="6">
+        <v>1</v>
+      </c>
+      <c r="O69" s="6">
         <v>99</v>
       </c>
-      <c r="O69" s="1">
-        <f>K69*L69*M69*N69</f>
+      <c r="P69" s="1">
+        <f t="shared" si="3"/>
         <v>198</v>
       </c>
-      <c r="P69" s="18"/>
       <c r="Q69" s="18"/>
       <c r="R69" s="18"/>
-    </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S69" s="18"/>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>52</v>
       </c>
@@ -4498,30 +4735,30 @@
       </c>
       <c r="C70" s="3"/>
       <c r="D70" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E70" s="5"/>
-      <c r="K70" s="1">
-        <v>1</v>
-      </c>
       <c r="L70" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M70" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N70" s="1">
+        <v>1</v>
+      </c>
+      <c r="O70" s="1">
         <v>5</v>
       </c>
-      <c r="O70" s="1">
-        <f>K70*L70*M70*N70</f>
+      <c r="P70" s="1">
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="P70" s="18"/>
       <c r="Q70" s="18"/>
       <c r="R70" s="18"/>
-    </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S70" s="18"/>
+    </row>
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>55</v>
       </c>
@@ -4529,36 +4766,33 @@
         <v>63</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J71" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="K71" s="1">
-        <v>2</v>
+      <c r="K71" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="L71" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M71" s="1">
         <v>1</v>
       </c>
       <c r="N71" s="1">
+        <v>1</v>
+      </c>
+      <c r="O71" s="1">
         <v>5</v>
       </c>
-      <c r="O71" s="1">
-        <f>K71*L71*M71*N71</f>
+      <c r="P71" s="1">
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="P71" s="25"/>
-      <c r="Q71" s="25"/>
-      <c r="R71" s="25"/>
-    </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>59</v>
       </c>
@@ -4566,37 +4800,34 @@
         <v>72</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E72" s="2"/>
-      <c r="K72" s="1">
-        <v>2</v>
-      </c>
       <c r="L72" s="1">
         <v>2</v>
       </c>
       <c r="M72" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N72" s="1">
+        <v>1</v>
+      </c>
+      <c r="O72" s="1">
         <v>5</v>
       </c>
-      <c r="O72" s="1">
-        <f>K72*L72*M72*N72</f>
+      <c r="P72" s="1">
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="P72" s="25"/>
-      <c r="Q72" s="25"/>
-      <c r="R72" s="25"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U72" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U72">
-      <sortCondition ref="Q1:Q72"/>
+  <autoFilter ref="A1:V72" xr:uid="{074061E7-583E-48EA-BC24-50BAFA208482}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V72">
+      <sortCondition ref="R1:R72"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="L2">
+  <conditionalFormatting sqref="M2">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="1"/>
@@ -4608,15 +4839,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S38">
+  <conditionalFormatting sqref="T2:T38">
     <cfRule type="expression" dxfId="2" priority="1">
-      <formula>$S2="L"</formula>
+      <formula>$T2="L"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$S2="H"</formula>
+      <formula>$T2="H"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="3">
-      <formula>$S2="-"</formula>
+      <formula>$T2="-"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>

</xml_diff>